<commit_message>
Adds facility capacity utilization plotting
Implements a new plotting function to visualize facility capacity utilization over time, broken down by location and technology.

This provides insights into how effectively facilities are being used and identifies potential bottlenecks or underutilized resources. The function generates plots showing both total and used capacity for each technology, enhancing understanding of capacity dynamics.

Also, enhance data processing to read and process facility-related data from Excel sheets. This includes reading data for facility capacity and utilization, ensuring accurate modeling of facility constraints and carryover effects within the URBS model.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF064698-A154-4B25-BE65-5FA2D3540356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED49FD0A-2C9F-4B91-B615-0332AE7669B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="-1935" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="60">
   <si>
     <t>Value</t>
   </si>
@@ -220,6 +220,9 @@
   </si>
   <si>
     <t>capacity_scrap_total</t>
+  </si>
+  <si>
+    <t>total_facility_cap_initial</t>
   </si>
 </sst>
 </file>
@@ -860,7 +863,7 @@
         <v>414000</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F2">
         <v>1775265.6417320003</v>
@@ -896,7 +899,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q2">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
@@ -913,7 +916,7 @@
         <v>414000</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F3">
         <v>1722922.372057667</v>
@@ -949,7 +952,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q3">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
@@ -966,7 +969,7 @@
         <v>414000</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F4">
         <v>1670579.1023833335</v>
@@ -1002,7 +1005,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q4">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
@@ -1019,7 +1022,7 @@
         <v>414000</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F5">
         <v>1618235.832709</v>
@@ -1055,7 +1058,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q5">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
@@ -1072,7 +1075,7 @@
         <v>414000</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F6">
         <v>1565892.5630346665</v>
@@ -1108,7 +1111,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q6">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
@@ -1125,7 +1128,7 @@
         <v>414000</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F7">
         <v>1513549.293360333</v>
@@ -1161,7 +1164,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q7">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
@@ -1178,7 +1181,7 @@
         <v>414000</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F8">
         <v>1461206.0236859999</v>
@@ -1214,7 +1217,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q8">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
@@ -1231,7 +1234,7 @@
         <v>414000</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F9">
         <v>1444015.15599508</v>
@@ -1267,7 +1270,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q9">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
@@ -1284,7 +1287,7 @@
         <v>414000</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F10">
         <v>1426824.2883041599</v>
@@ -1320,7 +1323,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q10">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
@@ -1337,7 +1340,7 @@
         <v>414000</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F11">
         <v>1409633.42061324</v>
@@ -1373,7 +1376,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q11">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
@@ -1390,7 +1393,7 @@
         <v>414000</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F12">
         <v>1392442.5529223196</v>
@@ -1426,7 +1429,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q12">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
@@ -1443,7 +1446,7 @@
         <v>414000</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F13">
         <v>1375251.6852313997</v>
@@ -1479,7 +1482,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q13">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
@@ -1496,7 +1499,7 @@
         <v>414000</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F14">
         <v>1358060.8175404796</v>
@@ -1532,7 +1535,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q14">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
@@ -1549,7 +1552,7 @@
         <v>414000</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F15">
         <v>1340869.9498495597</v>
@@ -1585,7 +1588,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q15">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
@@ -1602,7 +1605,7 @@
         <v>414000</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F16">
         <v>1323679.0821586396</v>
@@ -1638,7 +1641,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q16">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
@@ -1655,7 +1658,7 @@
         <v>414000</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F17">
         <v>1306488.2144677194</v>
@@ -1691,7 +1694,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q17">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
@@ -1708,7 +1711,7 @@
         <v>414000</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F18">
         <v>1288027.7959324</v>
@@ -1744,7 +1747,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q18">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
@@ -1761,7 +1764,7 @@
         <v>414000</v>
       </c>
       <c r="E19">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F19">
         <v>1288154.7510168403</v>
@@ -1797,7 +1800,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q19">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
@@ -1814,7 +1817,7 @@
         <v>414000</v>
       </c>
       <c r="E20">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F20">
         <v>1288281.7061012802</v>
@@ -1850,7 +1853,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q20">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.3">
@@ -1867,7 +1870,7 @@
         <v>414000</v>
       </c>
       <c r="E21">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F21">
         <v>1288408.6611857202</v>
@@ -1903,7 +1906,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q21">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
@@ -1920,7 +1923,7 @@
         <v>414000</v>
       </c>
       <c r="E22">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F22">
         <v>1288535.6162701603</v>
@@ -1956,7 +1959,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q22">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.3">
@@ -1973,7 +1976,7 @@
         <v>414000</v>
       </c>
       <c r="E23">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F23">
         <v>1288662.5713546001</v>
@@ -2009,7 +2012,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q23">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">
@@ -2026,7 +2029,7 @@
         <v>414000</v>
       </c>
       <c r="E24">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F24">
         <v>1288789.5264390404</v>
@@ -2062,7 +2065,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q24">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.3">
@@ -2079,7 +2082,7 @@
         <v>414000</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F25">
         <v>1288916.4815234803</v>
@@ -2115,7 +2118,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q25">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.3">
@@ -2132,7 +2135,7 @@
         <v>414000</v>
       </c>
       <c r="E26">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F26">
         <v>1289043.4366079206</v>
@@ -2168,7 +2171,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q26">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.3">
@@ -2185,7 +2188,7 @@
         <v>414000</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F27">
         <v>1289170.3916923604</v>
@@ -2221,7 +2224,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q27">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.3">
@@ -2238,7 +2241,7 @@
         <v>414000</v>
       </c>
       <c r="E28">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="F28">
         <v>1289297.3467768</v>
@@ -2274,7 +2277,7 @@
         <v>139589.9</v>
       </c>
       <c r="Q28">
-        <v>1</v>
+        <v>1000</v>
       </c>
     </row>
   </sheetData>
@@ -8865,7 +8868,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71493739-45C2-4A8D-9266-24BB3FC8F4DB}">
-  <dimension ref="A1:Z18"/>
+  <dimension ref="A1:AA18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.44140625" customWidth="1"/>
@@ -8879,7 +8882,7 @@
     <col min="20" max="20" width="20.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>18</v>
       </c>
@@ -8958,8 +8961,11 @@
       <c r="Z1" s="4" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA1" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
@@ -9038,8 +9044,11 @@
       <c r="Z2" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA2" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>31</v>
       </c>
@@ -9118,8 +9127,11 @@
       <c r="Z3" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA3" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>41</v>
       </c>
@@ -9198,8 +9210,11 @@
       <c r="Z4" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA4" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>56</v>
       </c>
@@ -9278,38 +9293,41 @@
       <c r="Z5" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="AA5" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" s="3"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Adds facility utilization plot and updates cost reductions
Adds a plot for facility utilization to the rolling horizon analysis.

Updates cost reduction parameters for wind, and adds cost reduction parameters for batteries.

Commented out facility utilization plot to prevent plot overlapping in standard plot function.
Enables debug prints for stockpile.py.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED49FD0A-2C9F-4B91-B615-0332AE7669B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFDECAE6-5F97-4137-9153-44686F3BABA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -860,10 +860,10 @@
         <v>303600</v>
       </c>
       <c r="D2">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F2">
         <v>1775265.6417320003</v>
@@ -872,10 +872,10 @@
         <v>2337972.5216000001</v>
       </c>
       <c r="H2">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J2">
         <v>1052044.8400000001</v>
@@ -884,10 +884,10 @@
         <v>1673707.7</v>
       </c>
       <c r="L2">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N2">
         <v>90210</v>
@@ -896,10 +896,10 @@
         <v>129380</v>
       </c>
       <c r="P2">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q2">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
@@ -913,10 +913,10 @@
         <v>299045.40000000002</v>
       </c>
       <c r="D3">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F3">
         <v>1722922.372057667</v>
@@ -925,10 +925,10 @@
         <v>2318026.381866667</v>
       </c>
       <c r="H3">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J3">
         <v>1042480.7960000001</v>
@@ -937,10 +937,10 @@
         <v>1660955.6413333334</v>
       </c>
       <c r="L3">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N3">
         <v>88856.85</v>
@@ -949,10 +949,10 @@
         <v>127438.3</v>
       </c>
       <c r="P3">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q3">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
@@ -966,10 +966,10 @@
         <v>294559.71899999998</v>
       </c>
       <c r="D4">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E4">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F4">
         <v>1670579.1023833335</v>
@@ -978,10 +978,10 @@
         <v>2298080.2421333333</v>
       </c>
       <c r="H4">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J4">
         <v>1032916.7520000001</v>
@@ -990,10 +990,10 @@
         <v>1648203.5826666667</v>
       </c>
       <c r="L4">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M4">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N4">
         <v>87523</v>
@@ -1002,10 +1002,10 @@
         <v>125526.73</v>
       </c>
       <c r="P4">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q4">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
@@ -1019,10 +1019,10 @@
         <v>290141.32319999998</v>
       </c>
       <c r="D5">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E5">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F5">
         <v>1618235.832709</v>
@@ -1031,10 +1031,10 @@
         <v>2278134.1023999997</v>
       </c>
       <c r="H5">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J5">
         <v>1023352.708</v>
@@ -1043,10 +1043,10 @@
         <v>1635451.524</v>
       </c>
       <c r="L5">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N5">
         <v>86209.15</v>
@@ -1055,10 +1055,10 @@
         <v>123644.83</v>
       </c>
       <c r="P5">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q5">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
@@ -1072,10 +1072,10 @@
         <v>285788.2034</v>
       </c>
       <c r="D6">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E6">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F6">
         <v>1565892.5630346665</v>
@@ -1084,10 +1084,10 @@
         <v>2258187.9626666661</v>
       </c>
       <c r="H6">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J6">
         <v>1013788.6639999999</v>
@@ -1096,10 +1096,10 @@
         <v>1622699.4653333335</v>
       </c>
       <c r="L6">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N6">
         <v>84915.01</v>
@@ -1108,10 +1108,10 @@
         <v>121792.16</v>
       </c>
       <c r="P6">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q6">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
@@ -1125,10 +1125,10 @@
         <v>281498.4804</v>
       </c>
       <c r="D7">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E7">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F7">
         <v>1513549.293360333</v>
@@ -1137,10 +1137,10 @@
         <v>2238241.8229333302</v>
       </c>
       <c r="H7">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J7">
         <v>1004224.62</v>
@@ -1149,10 +1149,10 @@
         <v>1609947.4066666667</v>
       </c>
       <c r="L7">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M7">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N7">
         <v>83640.289999999994</v>
@@ -1161,10 +1161,10 @@
         <v>119968.28</v>
       </c>
       <c r="P7">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q7">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
@@ -1178,10 +1178,10 @@
         <v>277270.34419999999</v>
       </c>
       <c r="D8">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E8">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F8">
         <v>1461206.0236859999</v>
@@ -1190,10 +1190,10 @@
         <v>2218295.6831999999</v>
       </c>
       <c r="H8">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J8">
         <v>994660.57600000012</v>
@@ -1202,10 +1202,10 @@
         <v>1597195.3480000002</v>
       </c>
       <c r="L8">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M8">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N8">
         <v>82384.69</v>
@@ -1214,10 +1214,10 @@
         <v>118172.75</v>
       </c>
       <c r="P8">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q8">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
@@ -1231,10 +1231,10 @@
         <v>273102.28909999999</v>
       </c>
       <c r="D9">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E9">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F9">
         <v>1444015.15599508</v>
@@ -1243,10 +1243,10 @@
         <v>2205259.4561600001</v>
       </c>
       <c r="H9">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J9">
         <v>992747.76720000012</v>
@@ -1255,10 +1255,10 @@
         <v>1594326.1348000003</v>
       </c>
       <c r="L9">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M9">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N9">
         <v>81147.92</v>
@@ -1267,10 +1267,10 @@
         <v>116405.16</v>
       </c>
       <c r="P9">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q9">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
@@ -1284,10 +1284,10 @@
         <v>268993.2548</v>
       </c>
       <c r="D10">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E10">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F10">
         <v>1426824.2883041599</v>
@@ -1296,10 +1296,10 @@
         <v>2192223.2291199998</v>
       </c>
       <c r="H10">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J10">
         <v>990834.9584</v>
@@ -1308,10 +1308,10 @@
         <v>1591456.9216000002</v>
       </c>
       <c r="L10">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M10">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N10">
         <v>79929.7</v>
@@ -1320,10 +1320,10 @@
         <v>114665.09</v>
       </c>
       <c r="P10">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q10">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
@@ -1337,10 +1337,10 @@
         <v>264942.41499999998</v>
       </c>
       <c r="D11">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E11">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F11">
         <v>1409633.42061324</v>
@@ -1349,10 +1349,10 @@
         <v>2179187.0020799995</v>
       </c>
       <c r="H11">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J11">
         <v>988922.1496</v>
@@ -1361,10 +1361,10 @@
         <v>1588587.7084000004</v>
       </c>
       <c r="L11">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M11">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N11">
         <v>78729.759999999995</v>
@@ -1373,10 +1373,10 @@
         <v>112952.12</v>
       </c>
       <c r="P11">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q11">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
@@ -1390,10 +1390,10 @@
         <v>260948.7948</v>
       </c>
       <c r="D12">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E12">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F12">
         <v>1392442.5529223196</v>
@@ -1402,10 +1402,10 @@
         <v>2166150.7750399997</v>
       </c>
       <c r="H12">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J12">
         <v>987009.34079999989</v>
@@ -1414,10 +1414,10 @@
         <v>1585718.4952000002</v>
       </c>
       <c r="L12">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M12">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N12">
         <v>77547.820000000007</v>
@@ -1426,10 +1426,10 @@
         <v>111265.84</v>
       </c>
       <c r="P12">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q12">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
@@ -1443,10 +1443,10 @@
         <v>257011.4613</v>
       </c>
       <c r="D13">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E13">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F13">
         <v>1375251.6852313997</v>
@@ -1455,10 +1455,10 @@
         <v>2153114.5479999995</v>
       </c>
       <c r="H13">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J13">
         <v>985096.53199999989</v>
@@ -1467,10 +1467,10 @@
         <v>1582849.2820000004</v>
       </c>
       <c r="L13">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M13">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N13">
         <v>76383.600000000006</v>
@@ -1479,10 +1479,10 @@
         <v>109605.86</v>
       </c>
       <c r="P13">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q13">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
@@ -1496,10 +1496,10 @@
         <v>253129.39139999999</v>
       </c>
       <c r="D14">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E14">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F14">
         <v>1358060.8175404796</v>
@@ -1508,10 +1508,10 @@
         <v>2140078.3209599997</v>
       </c>
       <c r="H14">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J14">
         <v>983183.72319999977</v>
@@ -1520,10 +1520,10 @@
         <v>1579980.0688000005</v>
       </c>
       <c r="L14">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M14">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N14">
         <v>75236.84</v>
@@ -1532,10 +1532,10 @@
         <v>107971.77</v>
       </c>
       <c r="P14">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q14">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
@@ -1549,10 +1549,10 @@
         <v>249301.63759999999</v>
       </c>
       <c r="D15">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E15">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F15">
         <v>1340869.9498495597</v>
@@ -1561,10 +1561,10 @@
         <v>2127042.0939199994</v>
       </c>
       <c r="H15">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J15">
         <v>981270.91439999978</v>
@@ -1573,10 +1573,10 @@
         <v>1577110.8556000004</v>
       </c>
       <c r="L15">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M15">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N15">
         <v>74107.289999999994</v>
@@ -1585,10 +1585,10 @@
         <v>106363.2</v>
       </c>
       <c r="P15">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q15">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
@@ -1602,10 +1602,10 @@
         <v>245527.30809999999</v>
       </c>
       <c r="D16">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E16">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F16">
         <v>1323679.0821586396</v>
@@ -1614,10 +1614,10 @@
         <v>2114005.8668799992</v>
       </c>
       <c r="H16">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J16">
         <v>979358.10559999966</v>
@@ -1626,10 +1626,10 @@
         <v>1574241.6424000005</v>
       </c>
       <c r="L16">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M16">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N16">
         <v>72994.679999999993</v>
@@ -1638,10 +1638,10 @@
         <v>104779.75</v>
       </c>
       <c r="P16">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q16">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
@@ -1655,10 +1655,10 @@
         <v>241805.39859999999</v>
       </c>
       <c r="D17">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E17">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F17">
         <v>1306488.2144677194</v>
@@ -1667,10 +1667,10 @@
         <v>2100969.6398399994</v>
       </c>
       <c r="H17">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J17">
         <v>977445.29679999966</v>
@@ -1679,10 +1679,10 @@
         <v>1571372.4292000004</v>
       </c>
       <c r="L17">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M17">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N17">
         <v>71898.759999999995</v>
@@ -1691,10 +1691,10 @@
         <v>103221.06</v>
       </c>
       <c r="P17">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q17">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
@@ -1708,10 +1708,10 @@
         <v>238134.9901</v>
       </c>
       <c r="D18">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E18">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F18">
         <v>1288027.7959324</v>
@@ -1720,10 +1720,10 @@
         <v>2087933.4128</v>
       </c>
       <c r="H18">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J18">
         <v>975532.48799999955</v>
@@ -1732,10 +1732,10 @@
         <v>1568503.2160000005</v>
       </c>
       <c r="L18">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M18">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N18">
         <v>70819.28</v>
@@ -1744,10 +1744,10 @@
         <v>101686.74</v>
       </c>
       <c r="P18">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q18">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
@@ -1761,10 +1761,10 @@
         <v>234515.065</v>
       </c>
       <c r="D19">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E19">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F19">
         <v>1288154.7510168403</v>
@@ -1773,10 +1773,10 @@
         <v>2076927.41784</v>
       </c>
       <c r="H19">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J19">
         <v>973619.67919999966</v>
@@ -1785,10 +1785,10 @@
         <v>1565634.0028000006</v>
       </c>
       <c r="L19">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M19">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N19">
         <v>69755.990000000005</v>
@@ -1797,10 +1797,10 @@
         <v>100176.44</v>
       </c>
       <c r="P19">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q19">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
@@ -1814,10 +1814,10 @@
         <v>230944.68799999999</v>
       </c>
       <c r="D20">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E20">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F20">
         <v>1288281.7061012802</v>
@@ -1826,10 +1826,10 @@
         <v>2065921.4228800002</v>
       </c>
       <c r="H20">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J20">
         <v>971706.87039999955</v>
@@ -1838,10 +1838,10 @@
         <v>1562764.7896000005</v>
       </c>
       <c r="L20">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M20">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N20">
         <v>68708.649999999994</v>
@@ -1850,10 +1850,10 @@
         <v>98689.79</v>
       </c>
       <c r="P20">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q20">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.3">
@@ -1867,10 +1867,10 @@
         <v>227422.96530000001</v>
       </c>
       <c r="D21">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E21">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F21">
         <v>1288408.6611857202</v>
@@ -1879,10 +1879,10 @@
         <v>2054915.4279200002</v>
       </c>
       <c r="H21">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I21">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J21">
         <v>969794.06159999955</v>
@@ -1891,10 +1891,10 @@
         <v>1559895.5764000006</v>
       </c>
       <c r="L21">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M21">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N21">
         <v>67677.02</v>
@@ -1903,10 +1903,10 @@
         <v>97226.44</v>
       </c>
       <c r="P21">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q21">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
@@ -1920,10 +1920,10 @@
         <v>223948.88099999999</v>
       </c>
       <c r="D22">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E22">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F22">
         <v>1288535.6162701603</v>
@@ -1932,10 +1932,10 @@
         <v>2043909.4329600004</v>
       </c>
       <c r="H22">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J22">
         <v>967881.25279999943</v>
@@ -1944,10 +1944,10 @@
         <v>1557026.3632000005</v>
       </c>
       <c r="L22">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M22">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N22">
         <v>66660.86</v>
@@ -1956,10 +1956,10 @@
         <v>95786.05</v>
       </c>
       <c r="P22">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q22">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.3">
@@ -1973,10 +1973,10 @@
         <v>220521.46350000001</v>
       </c>
       <c r="D23">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E23">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F23">
         <v>1288662.5713546001</v>
@@ -1985,10 +1985,10 @@
         <v>2032903.4380000005</v>
       </c>
       <c r="H23">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I23">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J23">
         <v>965968.44399999944</v>
@@ -1997,10 +1997,10 @@
         <v>1554157.1500000006</v>
       </c>
       <c r="L23">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M23">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N23">
         <v>65659.95</v>
@@ -2009,10 +2009,10 @@
         <v>94368.26</v>
       </c>
       <c r="P23">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q23">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">
@@ -2026,10 +2026,10 @@
         <v>217139.74350000001</v>
       </c>
       <c r="D24">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E24">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F24">
         <v>1288789.5264390404</v>
@@ -2038,10 +2038,10 @@
         <v>2021897.4430400007</v>
       </c>
       <c r="H24">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I24">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J24">
         <v>964055.63519999932</v>
@@ -2050,10 +2050,10 @@
         <v>1551287.9368000007</v>
       </c>
       <c r="L24">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M24">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N24">
         <v>64674.05</v>
@@ -2062,10 +2062,10 @@
         <v>92972.74</v>
       </c>
       <c r="P24">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q24">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.3">
@@ -2079,10 +2079,10 @@
         <v>213802.75769999999</v>
       </c>
       <c r="D25">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E25">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F25">
         <v>1288916.4815234803</v>
@@ -2091,10 +2091,10 @@
         <v>2010891.4480800009</v>
       </c>
       <c r="H25">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I25">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J25">
         <v>962142.82639999932</v>
@@ -2103,10 +2103,10 @@
         <v>1548418.7236000006</v>
       </c>
       <c r="L25">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M25">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N25">
         <v>63702.94</v>
@@ -2115,10 +2115,10 @@
         <v>91599.15</v>
       </c>
       <c r="P25">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q25">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.3">
@@ -2132,10 +2132,10 @@
         <v>210509.61679999999</v>
       </c>
       <c r="D26">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E26">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F26">
         <v>1289043.4366079206</v>
@@ -2144,10 +2144,10 @@
         <v>1999885.4531200009</v>
       </c>
       <c r="H26">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J26">
         <v>960230.01759999921</v>
@@ -2156,10 +2156,10 @@
         <v>1545549.5104000007</v>
       </c>
       <c r="L26">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M26">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N26">
         <v>62746.400000000001</v>
@@ -2168,10 +2168,10 @@
         <v>90247.16</v>
       </c>
       <c r="P26">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q26">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.3">
@@ -2185,10 +2185,10 @@
         <v>207259.3126</v>
       </c>
       <c r="D27">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E27">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F27">
         <v>1289170.3916923604</v>
@@ -2197,10 +2197,10 @@
         <v>1988879.4581600011</v>
       </c>
       <c r="H27">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I27">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J27">
         <v>958317.20879999921</v>
@@ -2209,10 +2209,10 @@
         <v>1542680.2972000006</v>
       </c>
       <c r="L27">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M27">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N27">
         <v>61804.2</v>
@@ -2221,10 +2221,10 @@
         <v>88916.45</v>
       </c>
       <c r="P27">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q27">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.3">
@@ -2238,10 +2238,10 @@
         <v>204050.9535</v>
       </c>
       <c r="D28">
-        <v>414000</v>
+        <v>368000</v>
       </c>
       <c r="E28">
-        <v>1000</v>
+        <v>988.8</v>
       </c>
       <c r="F28">
         <v>1289297.3467768</v>
@@ -2250,10 +2250,10 @@
         <v>1977873.4631999999</v>
       </c>
       <c r="H28">
-        <v>2380000</v>
+        <v>496000</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>12537.43</v>
       </c>
       <c r="J28">
         <v>956404.40000000026</v>
@@ -2262,10 +2262,10 @@
         <v>1539811.0840000003</v>
       </c>
       <c r="L28">
-        <v>1700000</v>
+        <v>496000</v>
       </c>
       <c r="M28">
-        <v>1</v>
+        <v>14114.8</v>
       </c>
       <c r="N28">
         <v>60876.14</v>
@@ -2274,10 +2274,10 @@
         <v>87606.7</v>
       </c>
       <c r="P28">
-        <v>139589.9</v>
+        <v>230000</v>
       </c>
       <c r="Q28">
-        <v>1000</v>
+        <v>6512.98</v>
       </c>
     </row>
   </sheetData>
@@ -9012,10 +9012,10 @@
         <v>5</v>
       </c>
       <c r="P2" s="6">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="Q2" s="6">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="R2" s="6">
         <v>0.85</v>
@@ -9095,10 +9095,10 @@
         <v>5</v>
       </c>
       <c r="P3" s="6">
-        <v>10000</v>
+        <v>150.27000000000001</v>
       </c>
       <c r="Q3" s="6">
-        <v>10000</v>
+        <v>150.27000000000001</v>
       </c>
       <c r="R3" s="6">
         <v>0.85</v>
@@ -9178,10 +9178,10 @@
         <v>5</v>
       </c>
       <c r="P4" s="6">
-        <v>10000</v>
+        <v>85.3</v>
       </c>
       <c r="Q4" s="6">
-        <v>10000</v>
+        <v>85.3</v>
       </c>
       <c r="R4" s="6">
         <v>0.85</v>
@@ -9243,7 +9243,7 @@
         <v>0.27439999999999998</v>
       </c>
       <c r="J5" s="6">
-        <v>0.27439999999999998</v>
+        <v>0.3</v>
       </c>
       <c r="K5" s="5">
         <v>0.8</v>

</xml_diff>

<commit_message>
Updates input data file
Updates the input Excel file with new data or modifications to existing data, likely to reflect the latest information needed for the application.
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFDECAE6-5F97-4137-9153-44686F3BABA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{150F7FBD-CA77-4252-8E4F-5DD69389CF9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="114">
   <si>
     <t>Value</t>
   </si>
@@ -223,6 +223,168 @@
   </si>
   <si>
     <t>total_facility_cap_initial</t>
+  </si>
+  <si>
+    <t>280 439,83</t>
+  </si>
+  <si>
+    <t>274 754,91</t>
+  </si>
+  <si>
+    <t>269 179,44</t>
+  </si>
+  <si>
+    <t>263 711,78</t>
+  </si>
+  <si>
+    <t>258 350,32</t>
+  </si>
+  <si>
+    <t>253 093,46</t>
+  </si>
+  <si>
+    <t>247 939,65</t>
+  </si>
+  <si>
+    <t>242 887,37</t>
+  </si>
+  <si>
+    <t>237 935,10</t>
+  </si>
+  <si>
+    <t>233 081,40</t>
+  </si>
+  <si>
+    <t>228 324,82</t>
+  </si>
+  <si>
+    <t>223 663,91</t>
+  </si>
+  <si>
+    <t>219 097,32</t>
+  </si>
+  <si>
+    <t>214 623,65</t>
+  </si>
+  <si>
+    <t>210 241,60</t>
+  </si>
+  <si>
+    <t>205 949,84</t>
+  </si>
+  <si>
+    <t>201 747,12</t>
+  </si>
+  <si>
+    <t>197 632,19</t>
+  </si>
+  <si>
+    <t>193 603,83</t>
+  </si>
+  <si>
+    <t>189 660,87</t>
+  </si>
+  <si>
+    <t>185 802,14</t>
+  </si>
+  <si>
+    <t>182 026,51</t>
+  </si>
+  <si>
+    <t>178 332,87</t>
+  </si>
+  <si>
+    <t>174 720,11</t>
+  </si>
+  <si>
+    <t>171 187,17</t>
+  </si>
+  <si>
+    <t>167 732,98</t>
+  </si>
+  <si>
+    <t>164 356,52</t>
+  </si>
+  <si>
+    <t>527 469,86</t>
+  </si>
+  <si>
+    <t>516 785,56</t>
+  </si>
+  <si>
+    <t>506 302,50</t>
+  </si>
+  <si>
+    <t>496 017,89</t>
+  </si>
+  <si>
+    <t>485 929,01</t>
+  </si>
+  <si>
+    <t>476 033,18</t>
+  </si>
+  <si>
+    <t>466 327,80</t>
+  </si>
+  <si>
+    <t>456 810,30</t>
+  </si>
+  <si>
+    <t>447 478,16</t>
+  </si>
+  <si>
+    <t>438 328,91</t>
+  </si>
+  <si>
+    <t>429 360,14</t>
+  </si>
+  <si>
+    <t>420 569,49</t>
+  </si>
+  <si>
+    <t>411 954,65</t>
+  </si>
+  <si>
+    <t>403 513,36</t>
+  </si>
+  <si>
+    <t>395 243,39</t>
+  </si>
+  <si>
+    <t>387 142,59</t>
+  </si>
+  <si>
+    <t>379 208,83</t>
+  </si>
+  <si>
+    <t>371 440,05</t>
+  </si>
+  <si>
+    <t>363 834,24</t>
+  </si>
+  <si>
+    <t>356 389,41</t>
+  </si>
+  <si>
+    <t>349 103,66</t>
+  </si>
+  <si>
+    <t>341 975,10</t>
+  </si>
+  <si>
+    <t>334 991,90</t>
+  </si>
+  <si>
+    <t>328 152,29</t>
+  </si>
+  <si>
+    <t>321 454,54</t>
+  </si>
+  <si>
+    <t>314 897,00</t>
+  </si>
+  <si>
+    <t>308 477,99</t>
   </si>
 </sst>
 </file>
@@ -791,6 +953,8 @@
     <col min="9" max="9" width="22.5546875" customWidth="1"/>
     <col min="10" max="10" width="24.109375" customWidth="1"/>
     <col min="11" max="11" width="27.6640625" customWidth="1"/>
+    <col min="12" max="12" width="22.88671875" customWidth="1"/>
+    <col min="13" max="13" width="20.109375" customWidth="1"/>
     <col min="15" max="15" width="32.77734375" customWidth="1"/>
     <col min="16" max="16" width="35.21875" customWidth="1"/>
     <col min="17" max="17" width="31.44140625" customWidth="1"/>
@@ -859,47 +1023,47 @@
       <c r="C2">
         <v>303600</v>
       </c>
-      <c r="D2">
-        <v>368000</v>
-      </c>
-      <c r="E2">
-        <v>988.8</v>
-      </c>
-      <c r="F2">
+      <c r="D2" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E2" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F2" s="8">
         <v>1775265.6417320003</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="8">
         <v>2337972.5216000001</v>
       </c>
-      <c r="H2">
-        <v>496000</v>
-      </c>
-      <c r="I2">
-        <v>12537.43</v>
-      </c>
-      <c r="J2">
+      <c r="H2" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I2" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J2" s="8">
         <v>1052044.8400000001</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="8">
         <v>1673707.7</v>
       </c>
-      <c r="L2">
-        <v>496000</v>
+      <c r="L2" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M2">
-        <v>14114.8</v>
-      </c>
-      <c r="N2">
-        <v>90210</v>
-      </c>
-      <c r="O2" s="8">
-        <v>129380</v>
-      </c>
-      <c r="P2">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="P2" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q2">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
@@ -912,47 +1076,47 @@
       <c r="C3">
         <v>299045.40000000002</v>
       </c>
-      <c r="D3">
-        <v>368000</v>
-      </c>
-      <c r="E3">
-        <v>988.8</v>
-      </c>
-      <c r="F3">
+      <c r="D3" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E3" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F3" s="8">
         <v>1722922.372057667</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="8">
         <v>2318026.381866667</v>
       </c>
-      <c r="H3">
-        <v>496000</v>
-      </c>
-      <c r="I3">
-        <v>12537.43</v>
-      </c>
-      <c r="J3">
+      <c r="H3" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I3" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J3" s="8">
         <v>1042480.7960000001</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="8">
         <v>1660955.6413333334</v>
       </c>
-      <c r="L3">
-        <v>496000</v>
+      <c r="L3" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M3">
-        <v>14114.8</v>
-      </c>
-      <c r="N3">
-        <v>88856.85</v>
-      </c>
-      <c r="O3" s="8">
-        <v>127438.3</v>
-      </c>
-      <c r="P3">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="P3" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q3">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
@@ -965,47 +1129,47 @@
       <c r="C4">
         <v>294559.71899999998</v>
       </c>
-      <c r="D4">
-        <v>368000</v>
-      </c>
-      <c r="E4">
-        <v>988.8</v>
-      </c>
-      <c r="F4">
+      <c r="D4" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E4" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F4" s="8">
         <v>1670579.1023833335</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="8">
         <v>2298080.2421333333</v>
       </c>
-      <c r="H4">
-        <v>496000</v>
-      </c>
-      <c r="I4">
-        <v>12537.43</v>
-      </c>
-      <c r="J4">
+      <c r="H4" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I4" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J4" s="8">
         <v>1032916.7520000001</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="8">
         <v>1648203.5826666667</v>
       </c>
-      <c r="L4">
-        <v>496000</v>
+      <c r="L4" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M4">
-        <v>14114.8</v>
-      </c>
-      <c r="N4">
-        <v>87523</v>
-      </c>
-      <c r="O4" s="8">
-        <v>125526.73</v>
-      </c>
-      <c r="P4">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="P4" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q4">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
@@ -1018,47 +1182,47 @@
       <c r="C5">
         <v>290141.32319999998</v>
       </c>
-      <c r="D5">
-        <v>368000</v>
-      </c>
-      <c r="E5">
-        <v>988.8</v>
-      </c>
-      <c r="F5">
+      <c r="D5" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E5" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F5" s="8">
         <v>1618235.832709</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="8">
         <v>2278134.1023999997</v>
       </c>
-      <c r="H5">
-        <v>496000</v>
-      </c>
-      <c r="I5">
-        <v>12537.43</v>
-      </c>
-      <c r="J5">
+      <c r="H5" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I5" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J5" s="8">
         <v>1023352.708</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="8">
         <v>1635451.524</v>
       </c>
-      <c r="L5">
-        <v>496000</v>
+      <c r="L5" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M5">
-        <v>14114.8</v>
-      </c>
-      <c r="N5">
-        <v>86209.15</v>
-      </c>
-      <c r="O5" s="8">
-        <v>123644.83</v>
-      </c>
-      <c r="P5">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="P5" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q5">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
@@ -1071,47 +1235,47 @@
       <c r="C6">
         <v>285788.2034</v>
       </c>
-      <c r="D6">
-        <v>368000</v>
-      </c>
-      <c r="E6">
-        <v>988.8</v>
-      </c>
-      <c r="F6">
+      <c r="D6" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E6" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F6" s="8">
         <v>1565892.5630346665</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="8">
         <v>2258187.9626666661</v>
       </c>
-      <c r="H6">
-        <v>496000</v>
-      </c>
-      <c r="I6">
-        <v>12537.43</v>
-      </c>
-      <c r="J6">
+      <c r="H6" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I6" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J6" s="8">
         <v>1013788.6639999999</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="8">
         <v>1622699.4653333335</v>
       </c>
-      <c r="L6">
-        <v>496000</v>
+      <c r="L6" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M6">
-        <v>14114.8</v>
-      </c>
-      <c r="N6">
-        <v>84915.01</v>
-      </c>
-      <c r="O6" s="8">
-        <v>121792.16</v>
-      </c>
-      <c r="P6">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="P6" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q6">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
@@ -1124,47 +1288,47 @@
       <c r="C7">
         <v>281498.4804</v>
       </c>
-      <c r="D7">
-        <v>368000</v>
-      </c>
-      <c r="E7">
-        <v>988.8</v>
-      </c>
-      <c r="F7">
+      <c r="D7" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E7" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F7" s="8">
         <v>1513549.293360333</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="8">
         <v>2238241.8229333302</v>
       </c>
-      <c r="H7">
-        <v>496000</v>
-      </c>
-      <c r="I7">
-        <v>12537.43</v>
-      </c>
-      <c r="J7">
+      <c r="H7" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I7" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J7" s="8">
         <v>1004224.62</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="8">
         <v>1609947.4066666667</v>
       </c>
-      <c r="L7">
-        <v>496000</v>
+      <c r="L7" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M7">
-        <v>14114.8</v>
-      </c>
-      <c r="N7">
-        <v>83640.289999999994</v>
-      </c>
-      <c r="O7" s="8">
-        <v>119968.28</v>
-      </c>
-      <c r="P7">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="P7" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q7">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
@@ -1177,47 +1341,47 @@
       <c r="C8">
         <v>277270.34419999999</v>
       </c>
-      <c r="D8">
-        <v>368000</v>
-      </c>
-      <c r="E8">
-        <v>988.8</v>
-      </c>
-      <c r="F8">
+      <c r="D8" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E8" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F8" s="8">
         <v>1461206.0236859999</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="8">
         <v>2218295.6831999999</v>
       </c>
-      <c r="H8">
-        <v>496000</v>
-      </c>
-      <c r="I8">
-        <v>12537.43</v>
-      </c>
-      <c r="J8">
+      <c r="H8" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I8" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J8" s="8">
         <v>994660.57600000012</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="8">
         <v>1597195.3480000002</v>
       </c>
-      <c r="L8">
-        <v>496000</v>
+      <c r="L8" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M8">
-        <v>14114.8</v>
-      </c>
-      <c r="N8">
-        <v>82384.69</v>
-      </c>
-      <c r="O8" s="8">
-        <v>118172.75</v>
-      </c>
-      <c r="P8">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="P8" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q8">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
@@ -1230,47 +1394,47 @@
       <c r="C9">
         <v>273102.28909999999</v>
       </c>
-      <c r="D9">
-        <v>368000</v>
-      </c>
-      <c r="E9">
-        <v>988.8</v>
-      </c>
-      <c r="F9">
+      <c r="D9" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E9" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F9" s="8">
         <v>1444015.15599508</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="8">
         <v>2205259.4561600001</v>
       </c>
-      <c r="H9">
-        <v>496000</v>
-      </c>
-      <c r="I9">
-        <v>12537.43</v>
-      </c>
-      <c r="J9">
+      <c r="H9" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I9" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J9" s="8">
         <v>992747.76720000012</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="8">
         <v>1594326.1348000003</v>
       </c>
-      <c r="L9">
-        <v>496000</v>
+      <c r="L9" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M9">
-        <v>14114.8</v>
-      </c>
-      <c r="N9">
-        <v>81147.92</v>
-      </c>
-      <c r="O9" s="8">
-        <v>116405.16</v>
-      </c>
-      <c r="P9">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="P9" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q9">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
@@ -1283,47 +1447,47 @@
       <c r="C10">
         <v>268993.2548</v>
       </c>
-      <c r="D10">
-        <v>368000</v>
-      </c>
-      <c r="E10">
-        <v>988.8</v>
-      </c>
-      <c r="F10">
+      <c r="D10" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E10" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F10" s="8">
         <v>1426824.2883041599</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="8">
         <v>2192223.2291199998</v>
       </c>
-      <c r="H10">
-        <v>496000</v>
-      </c>
-      <c r="I10">
-        <v>12537.43</v>
-      </c>
-      <c r="J10">
+      <c r="H10" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I10" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J10" s="8">
         <v>990834.9584</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="8">
         <v>1591456.9216000002</v>
       </c>
-      <c r="L10">
-        <v>496000</v>
+      <c r="L10" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M10">
-        <v>14114.8</v>
-      </c>
-      <c r="N10">
-        <v>79929.7</v>
-      </c>
-      <c r="O10" s="8">
-        <v>114665.09</v>
-      </c>
-      <c r="P10">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="P10" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q10">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
@@ -1336,47 +1500,47 @@
       <c r="C11">
         <v>264942.41499999998</v>
       </c>
-      <c r="D11">
-        <v>368000</v>
-      </c>
-      <c r="E11">
-        <v>988.8</v>
-      </c>
-      <c r="F11">
+      <c r="D11" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E11" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F11" s="8">
         <v>1409633.42061324</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="8">
         <v>2179187.0020799995</v>
       </c>
-      <c r="H11">
-        <v>496000</v>
-      </c>
-      <c r="I11">
-        <v>12537.43</v>
-      </c>
-      <c r="J11">
+      <c r="H11" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I11" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J11" s="8">
         <v>988922.1496</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="8">
         <v>1588587.7084000004</v>
       </c>
-      <c r="L11">
-        <v>496000</v>
+      <c r="L11" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M11">
-        <v>14114.8</v>
-      </c>
-      <c r="N11">
-        <v>78729.759999999995</v>
-      </c>
-      <c r="O11" s="8">
-        <v>112952.12</v>
-      </c>
-      <c r="P11">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="P11" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q11">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
@@ -1389,47 +1553,47 @@
       <c r="C12">
         <v>260948.7948</v>
       </c>
-      <c r="D12">
-        <v>368000</v>
-      </c>
-      <c r="E12">
-        <v>988.8</v>
-      </c>
-      <c r="F12">
+      <c r="D12" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E12" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F12" s="8">
         <v>1392442.5529223196</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="8">
         <v>2166150.7750399997</v>
       </c>
-      <c r="H12">
-        <v>496000</v>
-      </c>
-      <c r="I12">
-        <v>12537.43</v>
-      </c>
-      <c r="J12">
+      <c r="H12" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I12" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J12" s="8">
         <v>987009.34079999989</v>
       </c>
-      <c r="K12">
+      <c r="K12" s="8">
         <v>1585718.4952000002</v>
       </c>
-      <c r="L12">
-        <v>496000</v>
+      <c r="L12" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M12">
-        <v>14114.8</v>
-      </c>
-      <c r="N12">
-        <v>77547.820000000007</v>
-      </c>
-      <c r="O12" s="8">
-        <v>111265.84</v>
-      </c>
-      <c r="P12">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="O12" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="P12" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q12">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
@@ -1442,47 +1606,47 @@
       <c r="C13">
         <v>257011.4613</v>
       </c>
-      <c r="D13">
-        <v>368000</v>
-      </c>
-      <c r="E13">
-        <v>988.8</v>
-      </c>
-      <c r="F13">
+      <c r="D13" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E13" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F13" s="8">
         <v>1375251.6852313997</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="8">
         <v>2153114.5479999995</v>
       </c>
-      <c r="H13">
-        <v>496000</v>
-      </c>
-      <c r="I13">
-        <v>12537.43</v>
-      </c>
-      <c r="J13">
+      <c r="H13" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I13" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J13" s="8">
         <v>985096.53199999989</v>
       </c>
-      <c r="K13">
+      <c r="K13" s="8">
         <v>1582849.2820000004</v>
       </c>
-      <c r="L13">
-        <v>496000</v>
+      <c r="L13" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M13">
-        <v>14114.8</v>
-      </c>
-      <c r="N13">
-        <v>76383.600000000006</v>
-      </c>
-      <c r="O13" s="8">
-        <v>109605.86</v>
-      </c>
-      <c r="P13">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="P13" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q13">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
@@ -1495,47 +1659,47 @@
       <c r="C14">
         <v>253129.39139999999</v>
       </c>
-      <c r="D14">
-        <v>368000</v>
-      </c>
-      <c r="E14">
-        <v>988.8</v>
-      </c>
-      <c r="F14">
+      <c r="D14" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E14" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F14" s="8">
         <v>1358060.8175404796</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="8">
         <v>2140078.3209599997</v>
       </c>
-      <c r="H14">
-        <v>496000</v>
-      </c>
-      <c r="I14">
-        <v>12537.43</v>
-      </c>
-      <c r="J14">
+      <c r="H14" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I14" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J14" s="8">
         <v>983183.72319999977</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="8">
         <v>1579980.0688000005</v>
       </c>
-      <c r="L14">
-        <v>496000</v>
+      <c r="L14" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M14">
-        <v>14114.8</v>
-      </c>
-      <c r="N14">
-        <v>75236.84</v>
-      </c>
-      <c r="O14" s="8">
-        <v>107971.77</v>
-      </c>
-      <c r="P14">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="O14" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="P14" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q14">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
@@ -1548,47 +1712,47 @@
       <c r="C15">
         <v>249301.63759999999</v>
       </c>
-      <c r="D15">
-        <v>368000</v>
-      </c>
-      <c r="E15">
-        <v>988.8</v>
-      </c>
-      <c r="F15">
+      <c r="D15" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E15" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F15" s="8">
         <v>1340869.9498495597</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="8">
         <v>2127042.0939199994</v>
       </c>
-      <c r="H15">
-        <v>496000</v>
-      </c>
-      <c r="I15">
-        <v>12537.43</v>
-      </c>
-      <c r="J15">
+      <c r="H15" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I15" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J15" s="8">
         <v>981270.91439999978</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="8">
         <v>1577110.8556000004</v>
       </c>
-      <c r="L15">
-        <v>496000</v>
+      <c r="L15" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M15">
-        <v>14114.8</v>
-      </c>
-      <c r="N15">
-        <v>74107.289999999994</v>
-      </c>
-      <c r="O15">
-        <v>106363.2</v>
-      </c>
-      <c r="P15">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="P15" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q15">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
@@ -1601,47 +1765,47 @@
       <c r="C16">
         <v>245527.30809999999</v>
       </c>
-      <c r="D16">
-        <v>368000</v>
-      </c>
-      <c r="E16">
-        <v>988.8</v>
-      </c>
-      <c r="F16">
+      <c r="D16" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E16" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F16" s="8">
         <v>1323679.0821586396</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="8">
         <v>2114005.8668799992</v>
       </c>
-      <c r="H16">
-        <v>496000</v>
-      </c>
-      <c r="I16">
-        <v>12537.43</v>
-      </c>
-      <c r="J16">
+      <c r="H16" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I16" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J16" s="8">
         <v>979358.10559999966</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="8">
         <v>1574241.6424000005</v>
       </c>
-      <c r="L16">
-        <v>496000</v>
+      <c r="L16" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M16">
-        <v>14114.8</v>
-      </c>
-      <c r="N16">
-        <v>72994.679999999993</v>
-      </c>
-      <c r="O16">
-        <v>104779.75</v>
-      </c>
-      <c r="P16">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="P16" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q16">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
@@ -1654,47 +1818,47 @@
       <c r="C17">
         <v>241805.39859999999</v>
       </c>
-      <c r="D17">
-        <v>368000</v>
-      </c>
-      <c r="E17">
-        <v>988.8</v>
-      </c>
-      <c r="F17">
+      <c r="D17" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E17" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F17" s="8">
         <v>1306488.2144677194</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="8">
         <v>2100969.6398399994</v>
       </c>
-      <c r="H17">
-        <v>496000</v>
-      </c>
-      <c r="I17">
-        <v>12537.43</v>
-      </c>
-      <c r="J17">
+      <c r="H17" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I17" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J17" s="8">
         <v>977445.29679999966</v>
       </c>
-      <c r="K17">
+      <c r="K17" s="8">
         <v>1571372.4292000004</v>
       </c>
-      <c r="L17">
-        <v>496000</v>
+      <c r="L17" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M17">
-        <v>14114.8</v>
-      </c>
-      <c r="N17">
-        <v>71898.759999999995</v>
-      </c>
-      <c r="O17">
-        <v>103221.06</v>
-      </c>
-      <c r="P17">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="P17" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q17">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
@@ -1707,47 +1871,47 @@
       <c r="C18">
         <v>238134.9901</v>
       </c>
-      <c r="D18">
-        <v>368000</v>
-      </c>
-      <c r="E18">
-        <v>988.8</v>
-      </c>
-      <c r="F18">
+      <c r="D18" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E18" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F18" s="8">
         <v>1288027.7959324</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="8">
         <v>2087933.4128</v>
       </c>
-      <c r="H18">
-        <v>496000</v>
-      </c>
-      <c r="I18">
-        <v>12537.43</v>
-      </c>
-      <c r="J18">
+      <c r="H18" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I18" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J18" s="8">
         <v>975532.48799999955</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="8">
         <v>1568503.2160000005</v>
       </c>
-      <c r="L18">
-        <v>496000</v>
+      <c r="L18" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M18">
-        <v>14114.8</v>
-      </c>
-      <c r="N18">
-        <v>70819.28</v>
-      </c>
-      <c r="O18">
-        <v>101686.74</v>
-      </c>
-      <c r="P18">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="P18" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q18">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
@@ -1760,47 +1924,47 @@
       <c r="C19">
         <v>234515.065</v>
       </c>
-      <c r="D19">
-        <v>368000</v>
-      </c>
-      <c r="E19">
-        <v>988.8</v>
-      </c>
-      <c r="F19">
+      <c r="D19" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E19" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F19" s="8">
         <v>1288154.7510168403</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="8">
         <v>2076927.41784</v>
       </c>
-      <c r="H19">
-        <v>496000</v>
-      </c>
-      <c r="I19">
-        <v>12537.43</v>
-      </c>
-      <c r="J19">
+      <c r="H19" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I19" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J19" s="8">
         <v>973619.67919999966</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="8">
         <v>1565634.0028000006</v>
       </c>
-      <c r="L19">
-        <v>496000</v>
+      <c r="L19" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M19">
-        <v>14114.8</v>
-      </c>
-      <c r="N19">
-        <v>69755.990000000005</v>
-      </c>
-      <c r="O19">
-        <v>100176.44</v>
-      </c>
-      <c r="P19">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="O19" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="P19" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q19">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
@@ -1813,47 +1977,47 @@
       <c r="C20">
         <v>230944.68799999999</v>
       </c>
-      <c r="D20">
-        <v>368000</v>
-      </c>
-      <c r="E20">
-        <v>988.8</v>
-      </c>
-      <c r="F20">
+      <c r="D20" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E20" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F20" s="8">
         <v>1288281.7061012802</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="8">
         <v>2065921.4228800002</v>
       </c>
-      <c r="H20">
-        <v>496000</v>
-      </c>
-      <c r="I20">
-        <v>12537.43</v>
-      </c>
-      <c r="J20">
+      <c r="H20" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I20" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J20" s="8">
         <v>971706.87039999955</v>
       </c>
-      <c r="K20">
+      <c r="K20" s="8">
         <v>1562764.7896000005</v>
       </c>
-      <c r="L20">
-        <v>496000</v>
+      <c r="L20" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M20">
-        <v>14114.8</v>
-      </c>
-      <c r="N20">
-        <v>68708.649999999994</v>
-      </c>
-      <c r="O20">
-        <v>98689.79</v>
-      </c>
-      <c r="P20">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N20" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="O20" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="P20" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q20">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.3">
@@ -1866,47 +2030,47 @@
       <c r="C21">
         <v>227422.96530000001</v>
       </c>
-      <c r="D21">
-        <v>368000</v>
-      </c>
-      <c r="E21">
-        <v>988.8</v>
-      </c>
-      <c r="F21">
+      <c r="D21" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E21" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F21" s="8">
         <v>1288408.6611857202</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="8">
         <v>2054915.4279200002</v>
       </c>
-      <c r="H21">
-        <v>496000</v>
-      </c>
-      <c r="I21">
-        <v>12537.43</v>
-      </c>
-      <c r="J21">
+      <c r="H21" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I21" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J21" s="8">
         <v>969794.06159999955</v>
       </c>
-      <c r="K21">
+      <c r="K21" s="8">
         <v>1559895.5764000006</v>
       </c>
-      <c r="L21">
-        <v>496000</v>
+      <c r="L21" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M21">
-        <v>14114.8</v>
-      </c>
-      <c r="N21">
-        <v>67677.02</v>
-      </c>
-      <c r="O21">
-        <v>97226.44</v>
-      </c>
-      <c r="P21">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="O21" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="P21" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q21">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
@@ -1919,47 +2083,47 @@
       <c r="C22">
         <v>223948.88099999999</v>
       </c>
-      <c r="D22">
-        <v>368000</v>
-      </c>
-      <c r="E22">
-        <v>988.8</v>
-      </c>
-      <c r="F22">
+      <c r="D22" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E22" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F22" s="8">
         <v>1288535.6162701603</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="8">
         <v>2043909.4329600004</v>
       </c>
-      <c r="H22">
-        <v>496000</v>
-      </c>
-      <c r="I22">
-        <v>12537.43</v>
-      </c>
-      <c r="J22">
+      <c r="H22" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I22" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J22" s="8">
         <v>967881.25279999943</v>
       </c>
-      <c r="K22">
+      <c r="K22" s="8">
         <v>1557026.3632000005</v>
       </c>
-      <c r="L22">
-        <v>496000</v>
+      <c r="L22" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M22">
-        <v>14114.8</v>
-      </c>
-      <c r="N22">
-        <v>66660.86</v>
-      </c>
-      <c r="O22">
-        <v>95786.05</v>
-      </c>
-      <c r="P22">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="O22" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="P22" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q22">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.3">
@@ -1972,47 +2136,47 @@
       <c r="C23">
         <v>220521.46350000001</v>
       </c>
-      <c r="D23">
-        <v>368000</v>
-      </c>
-      <c r="E23">
-        <v>988.8</v>
-      </c>
-      <c r="F23">
+      <c r="D23" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E23" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F23" s="8">
         <v>1288662.5713546001</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="8">
         <v>2032903.4380000005</v>
       </c>
-      <c r="H23">
-        <v>496000</v>
-      </c>
-      <c r="I23">
-        <v>12537.43</v>
-      </c>
-      <c r="J23">
+      <c r="H23" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I23" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J23" s="8">
         <v>965968.44399999944</v>
       </c>
-      <c r="K23">
+      <c r="K23" s="8">
         <v>1554157.1500000006</v>
       </c>
-      <c r="L23">
-        <v>496000</v>
+      <c r="L23" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M23">
-        <v>14114.8</v>
-      </c>
-      <c r="N23">
-        <v>65659.95</v>
-      </c>
-      <c r="O23">
-        <v>94368.26</v>
-      </c>
-      <c r="P23">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N23" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="O23" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="P23" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q23">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">
@@ -2025,47 +2189,47 @@
       <c r="C24">
         <v>217139.74350000001</v>
       </c>
-      <c r="D24">
-        <v>368000</v>
-      </c>
-      <c r="E24">
-        <v>988.8</v>
-      </c>
-      <c r="F24">
+      <c r="D24" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E24" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F24" s="8">
         <v>1288789.5264390404</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="8">
         <v>2021897.4430400007</v>
       </c>
-      <c r="H24">
-        <v>496000</v>
-      </c>
-      <c r="I24">
-        <v>12537.43</v>
-      </c>
-      <c r="J24">
+      <c r="H24" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I24" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J24" s="8">
         <v>964055.63519999932</v>
       </c>
-      <c r="K24">
+      <c r="K24" s="8">
         <v>1551287.9368000007</v>
       </c>
-      <c r="L24">
-        <v>496000</v>
+      <c r="L24" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M24">
-        <v>14114.8</v>
-      </c>
-      <c r="N24">
-        <v>64674.05</v>
-      </c>
-      <c r="O24">
-        <v>92972.74</v>
-      </c>
-      <c r="P24">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="O24" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="P24" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q24">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.3">
@@ -2078,47 +2242,47 @@
       <c r="C25">
         <v>213802.75769999999</v>
       </c>
-      <c r="D25">
-        <v>368000</v>
-      </c>
-      <c r="E25">
-        <v>988.8</v>
-      </c>
-      <c r="F25">
+      <c r="D25" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E25" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F25" s="8">
         <v>1288916.4815234803</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="8">
         <v>2010891.4480800009</v>
       </c>
-      <c r="H25">
-        <v>496000</v>
-      </c>
-      <c r="I25">
-        <v>12537.43</v>
-      </c>
-      <c r="J25">
+      <c r="H25" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I25" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J25" s="8">
         <v>962142.82639999932</v>
       </c>
-      <c r="K25">
+      <c r="K25" s="8">
         <v>1548418.7236000006</v>
       </c>
-      <c r="L25">
-        <v>496000</v>
+      <c r="L25" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M25">
-        <v>14114.8</v>
-      </c>
-      <c r="N25">
-        <v>63702.94</v>
-      </c>
-      <c r="O25">
-        <v>91599.15</v>
-      </c>
-      <c r="P25">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N25" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="O25" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="P25" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q25">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.3">
@@ -2131,47 +2295,47 @@
       <c r="C26">
         <v>210509.61679999999</v>
       </c>
-      <c r="D26">
-        <v>368000</v>
-      </c>
-      <c r="E26">
-        <v>988.8</v>
-      </c>
-      <c r="F26">
+      <c r="D26" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E26" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F26" s="8">
         <v>1289043.4366079206</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="8">
         <v>1999885.4531200009</v>
       </c>
-      <c r="H26">
-        <v>496000</v>
-      </c>
-      <c r="I26">
-        <v>12537.43</v>
-      </c>
-      <c r="J26">
+      <c r="H26" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I26" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J26" s="8">
         <v>960230.01759999921</v>
       </c>
-      <c r="K26">
+      <c r="K26" s="8">
         <v>1545549.5104000007</v>
       </c>
-      <c r="L26">
-        <v>496000</v>
+      <c r="L26" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M26">
-        <v>14114.8</v>
-      </c>
-      <c r="N26">
-        <v>62746.400000000001</v>
-      </c>
-      <c r="O26">
-        <v>90247.16</v>
-      </c>
-      <c r="P26">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="O26" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="P26" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q26">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.3">
@@ -2184,47 +2348,47 @@
       <c r="C27">
         <v>207259.3126</v>
       </c>
-      <c r="D27">
-        <v>368000</v>
-      </c>
-      <c r="E27">
-        <v>988.8</v>
-      </c>
-      <c r="F27">
+      <c r="D27" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E27" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F27" s="8">
         <v>1289170.3916923604</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="8">
         <v>1988879.4581600011</v>
       </c>
-      <c r="H27">
-        <v>496000</v>
-      </c>
-      <c r="I27">
-        <v>12537.43</v>
-      </c>
-      <c r="J27">
+      <c r="H27" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I27" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J27" s="8">
         <v>958317.20879999921</v>
       </c>
-      <c r="K27">
+      <c r="K27" s="8">
         <v>1542680.2972000006</v>
       </c>
-      <c r="L27">
-        <v>496000</v>
+      <c r="L27" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M27">
-        <v>14114.8</v>
-      </c>
-      <c r="N27">
-        <v>61804.2</v>
-      </c>
-      <c r="O27">
-        <v>88916.45</v>
-      </c>
-      <c r="P27">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N27" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="O27" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="P27" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q27">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.3">
@@ -2237,47 +2401,47 @@
       <c r="C28">
         <v>204050.9535</v>
       </c>
-      <c r="D28">
-        <v>368000</v>
-      </c>
-      <c r="E28">
-        <v>988.8</v>
-      </c>
-      <c r="F28">
+      <c r="D28" s="8">
+        <v>227700</v>
+      </c>
+      <c r="E28" s="8">
+        <v>1000</v>
+      </c>
+      <c r="F28" s="8">
         <v>1289297.3467768</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="8">
         <v>1977873.4631999999</v>
       </c>
-      <c r="H28">
-        <v>496000</v>
-      </c>
-      <c r="I28">
-        <v>12537.43</v>
-      </c>
-      <c r="J28">
+      <c r="H28" s="8">
+        <v>1646946.1610000001</v>
+      </c>
+      <c r="I28" s="8">
+        <v>1000</v>
+      </c>
+      <c r="J28" s="8">
         <v>956404.40000000026</v>
       </c>
-      <c r="K28">
+      <c r="K28" s="8">
         <v>1539811.0840000003</v>
       </c>
-      <c r="L28">
-        <v>496000</v>
+      <c r="L28" s="8">
+        <v>1093231.041</v>
       </c>
       <c r="M28">
-        <v>14114.8</v>
-      </c>
-      <c r="N28">
-        <v>60876.14</v>
-      </c>
-      <c r="O28">
-        <v>87606.7</v>
-      </c>
-      <c r="P28">
-        <v>230000</v>
+        <v>1000</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="O28" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="P28" s="8">
+        <v>489061.86</v>
       </c>
       <c r="Q28">
-        <v>6512.98</v>
+        <v>1000</v>
       </c>
     </row>
   </sheetData>
@@ -8985,7 +9149,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="6">
-        <v>1500</v>
+        <v>13000</v>
       </c>
       <c r="H2" s="5">
         <v>0</v>
@@ -9012,10 +9176,10 @@
         <v>5</v>
       </c>
       <c r="P2" s="6">
-        <v>90</v>
+        <v>76.923000000000002</v>
       </c>
       <c r="Q2" s="6">
-        <v>90</v>
+        <v>76.923000000000002</v>
       </c>
       <c r="R2" s="6">
         <v>0.85</v>
@@ -9095,13 +9259,13 @@
         <v>5</v>
       </c>
       <c r="P3" s="6">
-        <v>150.27000000000001</v>
+        <v>126.83</v>
       </c>
       <c r="Q3" s="6">
-        <v>150.27000000000001</v>
+        <v>126.83</v>
       </c>
       <c r="R3" s="6">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S3" s="6">
         <v>0.2</v>
@@ -9178,13 +9342,13 @@
         <v>5</v>
       </c>
       <c r="P4" s="6">
-        <v>85.3</v>
+        <v>126.83</v>
       </c>
       <c r="Q4" s="6">
-        <v>85.3</v>
+        <v>126.83</v>
       </c>
       <c r="R4" s="6">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="S4" s="6">
         <v>0.2</v>

</xml_diff>

<commit_message>
disenabled prucereduction on scrap
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FA2D59B-8BB7-4815-BB60-5AF9193FB5FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7503729A-C057-4E46-ADEE-6887F65A1064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="7" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -544,7 +544,7 @@
     </xf>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -562,6 +562,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{1C1ADB5D-62B2-4A88-A962-14B0B3D457AA}"/>
@@ -10512,13 +10513,13 @@
         <v>2024</v>
       </c>
       <c r="B2">
-        <v>70000</v>
-      </c>
-      <c r="C2">
-        <v>26250</v>
-      </c>
-      <c r="D2">
-        <v>36915</v>
+        <v>65.5</v>
+      </c>
+      <c r="C2" s="9">
+        <v>2.1</v>
+      </c>
+      <c r="D2" s="9">
+        <v>15.28</v>
       </c>
       <c r="E2">
         <v>999999</v>
@@ -10529,13 +10530,14 @@
         <v>2025</v>
       </c>
       <c r="B3">
-        <v>70000</v>
-      </c>
-      <c r="C3">
-        <v>26250</v>
-      </c>
-      <c r="D3">
-        <v>36915</v>
+        <f>SUM(B2*1.04)</f>
+        <v>68.12</v>
+      </c>
+      <c r="C3" s="9">
+        <v>2.1</v>
+      </c>
+      <c r="D3" s="9">
+        <v>15.28</v>
       </c>
       <c r="E3">
         <v>999999</v>
@@ -10546,13 +10548,14 @@
         <v>2026</v>
       </c>
       <c r="B4">
-        <v>70000</v>
-      </c>
-      <c r="C4">
-        <v>26250</v>
-      </c>
-      <c r="D4">
-        <v>36915</v>
+        <f t="shared" ref="B4:B9" si="0">SUM(B3*1.04)</f>
+        <v>70.844800000000006</v>
+      </c>
+      <c r="C4" s="9">
+        <v>3.96</v>
+      </c>
+      <c r="D4" s="9">
+        <v>15.85</v>
       </c>
       <c r="E4">
         <v>999999</v>
@@ -10563,13 +10566,14 @@
         <v>2027</v>
       </c>
       <c r="B5">
-        <v>70000</v>
-      </c>
-      <c r="C5">
-        <v>26250</v>
-      </c>
-      <c r="D5">
-        <v>36915</v>
+        <f t="shared" si="0"/>
+        <v>73.678592000000009</v>
+      </c>
+      <c r="C5" s="9">
+        <v>3.42</v>
+      </c>
+      <c r="D5" s="9">
+        <v>18.7</v>
       </c>
       <c r="E5">
         <v>999999</v>
@@ -10580,13 +10584,14 @@
         <v>2028</v>
       </c>
       <c r="B6">
-        <v>70000</v>
-      </c>
-      <c r="C6">
-        <v>26250</v>
-      </c>
-      <c r="D6">
-        <v>36915</v>
+        <f t="shared" si="0"/>
+        <v>76.625735680000005</v>
+      </c>
+      <c r="C6" s="9">
+        <v>4.99</v>
+      </c>
+      <c r="D6" s="9">
+        <v>20.440000000000001</v>
       </c>
       <c r="E6">
         <v>999999</v>
@@ -10597,13 +10602,14 @@
         <v>2029</v>
       </c>
       <c r="B7">
-        <v>70000</v>
-      </c>
-      <c r="C7">
-        <v>26250</v>
-      </c>
-      <c r="D7">
-        <v>36915</v>
+        <f t="shared" si="0"/>
+        <v>79.690765107200008</v>
+      </c>
+      <c r="C7" s="9">
+        <v>6.41</v>
+      </c>
+      <c r="D7" s="9">
+        <v>20.9</v>
       </c>
       <c r="E7">
         <v>999999</v>
@@ -10614,13 +10620,14 @@
         <v>2030</v>
       </c>
       <c r="B8">
-        <v>70000</v>
-      </c>
-      <c r="C8">
-        <v>26250</v>
-      </c>
-      <c r="D8">
-        <v>21800</v>
+        <f t="shared" si="0"/>
+        <v>82.878395711488011</v>
+      </c>
+      <c r="C8" s="9">
+        <v>6.31</v>
+      </c>
+      <c r="D8" s="9">
+        <v>21.8</v>
       </c>
       <c r="E8">
         <v>999999</v>
@@ -10631,13 +10638,15 @@
         <v>2031</v>
       </c>
       <c r="B9">
-        <v>70000</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C9">
-        <v>26250</v>
+        <f>SUM(C8*1.2465)</f>
+        <v>7.8654149999999987</v>
       </c>
       <c r="D9">
-        <v>21800</v>
+        <f>SUM(D8*1.0626)</f>
+        <v>23.164680000000001</v>
       </c>
       <c r="E9">
         <v>999999</v>
@@ -10648,13 +10657,15 @@
         <v>2032</v>
       </c>
       <c r="B10">
-        <v>70000</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C10">
-        <v>26250</v>
+        <f t="shared" ref="C10:C12" si="1">SUM(C9*1.2465)</f>
+        <v>9.8042397974999975</v>
       </c>
       <c r="D10">
-        <v>21800</v>
+        <f t="shared" ref="D10:D13" si="2">SUM(D9*1.0626)</f>
+        <v>24.614788967999999</v>
       </c>
       <c r="E10">
         <v>999999</v>
@@ -10665,13 +10676,15 @@
         <v>2033</v>
       </c>
       <c r="B11">
-        <v>70000</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C11">
-        <v>26250</v>
+        <f t="shared" si="1"/>
+        <v>12.220984907583746</v>
       </c>
       <c r="D11">
-        <v>21800</v>
+        <f t="shared" si="2"/>
+        <v>26.155674757396799</v>
       </c>
       <c r="E11">
         <v>999999</v>
@@ -10682,13 +10695,15 @@
         <v>2034</v>
       </c>
       <c r="B12">
-        <v>70000</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C12">
-        <v>26250</v>
+        <f t="shared" si="1"/>
+        <v>15.233457687303138</v>
       </c>
       <c r="D12">
-        <v>21800</v>
+        <f t="shared" si="2"/>
+        <v>27.793019997209839</v>
       </c>
       <c r="E12">
         <v>999999</v>
@@ -10699,13 +10714,15 @@
         <v>2035</v>
       </c>
       <c r="B13">
-        <v>70000</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C13">
-        <v>26250</v>
+        <f>SUM(C12*1.2465)</f>
+        <v>18.98850500722336</v>
       </c>
       <c r="D13">
-        <v>21800</v>
+        <f t="shared" si="2"/>
+        <v>29.532863049035175</v>
       </c>
       <c r="E13">
         <v>999999</v>
@@ -10716,13 +10733,13 @@
         <v>2036</v>
       </c>
       <c r="B14">
-        <v>70000</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C14">
-        <v>26250</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D14">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E14">
         <v>999999</v>
@@ -10733,13 +10750,13 @@
         <v>2037</v>
       </c>
       <c r="B15">
-        <v>70000</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C15">
-        <v>26250</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D15">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E15">
         <v>999999</v>
@@ -10750,13 +10767,13 @@
         <v>2038</v>
       </c>
       <c r="B16">
-        <v>70000</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C16">
-        <v>26250</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D16">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E16">
         <v>999999</v>
@@ -10767,13 +10784,13 @@
         <v>2039</v>
       </c>
       <c r="B17">
-        <v>70000</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C17">
-        <v>26250</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D17">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E17">
         <v>999999</v>
@@ -10784,13 +10801,13 @@
         <v>2040</v>
       </c>
       <c r="B18">
-        <v>58400</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C18">
-        <v>18000</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D18">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E18">
         <v>999999</v>
@@ -10801,13 +10818,13 @@
         <v>2041</v>
       </c>
       <c r="B19">
-        <v>58400</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C19">
-        <v>18000</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D19">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E19">
         <v>999999</v>
@@ -10818,13 +10835,13 @@
         <v>2042</v>
       </c>
       <c r="B20">
-        <v>58400</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C20">
-        <v>18000</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D20">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E20">
         <v>999999</v>
@@ -10835,13 +10852,13 @@
         <v>2043</v>
       </c>
       <c r="B21">
-        <v>58400</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C21">
-        <v>18000</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D21">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E21">
         <v>999999</v>
@@ -10852,13 +10869,13 @@
         <v>2044</v>
       </c>
       <c r="B22">
-        <v>58400</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C22">
-        <v>18000</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D22">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E22">
         <v>999999</v>
@@ -10869,13 +10886,13 @@
         <v>2045</v>
       </c>
       <c r="B23">
-        <v>58400</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C23">
-        <v>18000</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D23">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E23">
         <v>999999</v>
@@ -10886,13 +10903,13 @@
         <v>2046</v>
       </c>
       <c r="B24">
-        <v>58400</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C24">
-        <v>18000</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D24">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E24">
         <v>999999</v>
@@ -10903,13 +10920,13 @@
         <v>2047</v>
       </c>
       <c r="B25">
-        <v>58400</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C25">
-        <v>18000</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D25">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E25">
         <v>999999</v>
@@ -10920,13 +10937,13 @@
         <v>2048</v>
       </c>
       <c r="B26">
-        <v>58400</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C26">
-        <v>18000</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D26">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E26">
         <v>999999</v>
@@ -10937,13 +10954,13 @@
         <v>2049</v>
       </c>
       <c r="B27">
-        <v>58400</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C27">
-        <v>18000</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D27">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E27">
         <v>999999</v>
@@ -10954,13 +10971,13 @@
         <v>2050</v>
       </c>
       <c r="B28">
-        <v>58400</v>
+        <v>82.878395711488011</v>
       </c>
       <c r="C28">
-        <v>18000</v>
+        <v>18.98850500722336</v>
       </c>
       <c r="D28">
-        <v>21800</v>
+        <v>29.532863049035175</v>
       </c>
       <c r="E28">
         <v>999999</v>

</xml_diff>

<commit_message>
edited scrap wind to 118t/MW
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8A0B217-3077-4B04-8989-9088753CD6B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C018DE9-0399-4D28-8BD4-9DD518F7785D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="7" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="67080" yWindow="-1935" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -9266,10 +9266,10 @@
         <v>5</v>
       </c>
       <c r="P3" s="6">
-        <v>126.83</v>
+        <v>118</v>
       </c>
       <c r="Q3" s="6">
-        <v>126.83</v>
+        <v>118</v>
       </c>
       <c r="R3" s="6">
         <v>0.95</v>
@@ -9349,10 +9349,10 @@
         <v>5</v>
       </c>
       <c r="P4" s="6">
-        <v>126.83</v>
+        <v>118</v>
       </c>
       <c r="Q4" s="6">
-        <v>126.83</v>
+        <v>118</v>
       </c>
       <c r="R4" s="6">
         <v>0.95</v>
@@ -10547,7 +10547,7 @@
         <v>2026</v>
       </c>
       <c r="B4">
-        <f t="shared" ref="B4:B9" si="0">SUM(B3*1.04)</f>
+        <f t="shared" ref="B4:B8" si="0">SUM(B3*1.04)</f>
         <v>70844.800000000003</v>
       </c>
       <c r="C4">

</xml_diff>

<commit_message>
there was a problem with urbs_extension specific params!
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C018DE9-0399-4D28-8BD4-9DD518F7785D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76775CF2-2FE5-492A-BD98-4162FA4A53CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="-1935" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="67080" yWindow="-5565" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -544,7 +544,7 @@
     </xf>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -562,6 +562,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma 2" xfId="2" xr:uid="{1C1ADB5D-62B2-4A88-A962-14B0B3D457AA}"/>
@@ -9339,7 +9342,7 @@
       <c r="L4" s="5">
         <v>0.2</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="9">
         <v>20</v>
       </c>
       <c r="N4" s="5">

</xml_diff>

<commit_message>
added via different route through res_vertex. Results not that convincing yet
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1F0D3AF-A98A-465D-816D-3782FCA9A9BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1294A14-454B-4C12-A610-4EBC208C09E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
@@ -23,6 +23,9 @@
     <sheet name="installable_capacity" sheetId="3" r:id="rId8"/>
     <sheet name="lng_block" sheetId="13" r:id="rId9"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">lng_block!$C$1:$C$15</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -632,7 +635,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -9241,10 +9244,10 @@
         <v>0.38879999999999998</v>
       </c>
       <c r="K2" s="5">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="L2" s="5">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="M2">
         <v>25</v>
@@ -9324,10 +9327,10 @@
         <v>0.2</v>
       </c>
       <c r="K3" s="5">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="L3" s="5">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="M3">
         <v>20</v>
@@ -9407,10 +9410,10 @@
         <v>0.2</v>
       </c>
       <c r="K4" s="5">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="L4" s="5">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="M4" s="9">
         <v>20</v>
@@ -9490,10 +9493,10 @@
         <v>0.3</v>
       </c>
       <c r="K5" s="5">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="L5" s="5">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="M5">
         <v>30</v>
@@ -10713,11 +10716,9 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C9">
-        <f>SUM(C8*1.2465)</f>
-        <v>7865.415</v>
+        <v>7865.4149999999991</v>
       </c>
       <c r="D9">
-        <f>SUM(D8*1.0626)</f>
         <v>23164.68</v>
       </c>
       <c r="E9">
@@ -10732,11 +10733,9 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C10">
-        <f t="shared" ref="C10:C12" si="1">SUM(C9*1.2465)</f>
-        <v>9804.2397975000003</v>
+        <v>9804.2397974999967</v>
       </c>
       <c r="D10">
-        <f t="shared" ref="D10:D13" si="2">SUM(D9*1.0626)</f>
         <v>24614.788968000001</v>
       </c>
       <c r="E10">
@@ -10751,12 +10750,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C11">
-        <f t="shared" si="1"/>
-        <v>12220.98490758375</v>
+        <v>12220.984907583746</v>
       </c>
       <c r="D11">
-        <f t="shared" si="2"/>
-        <v>26155.674757396802</v>
+        <v>26155.674757396799</v>
       </c>
       <c r="E11">
         <v>999999</v>
@@ -10770,12 +10767,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C12">
-        <f t="shared" si="1"/>
-        <v>15233.457687303144</v>
+        <v>15233.457687303138</v>
       </c>
       <c r="D12">
-        <f t="shared" si="2"/>
-        <v>27793.019997209842</v>
+        <v>27793.019997209838</v>
       </c>
       <c r="E12">
         <v>999999</v>
@@ -10789,12 +10784,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C13">
-        <f>SUM(C12*1.2465)</f>
-        <v>18988.505007223368</v>
+        <v>18988.505007223361</v>
       </c>
       <c r="D13">
-        <f t="shared" si="2"/>
-        <v>29532.863049035179</v>
+        <v>29532.863049035175</v>
       </c>
       <c r="E13">
         <v>999999</v>
@@ -10808,10 +10801,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C14">
-        <v>18988.505007223368</v>
+        <v>20887.355507945696</v>
       </c>
       <c r="D14">
-        <v>29532.863049035179</v>
+        <v>29532.863049035175</v>
       </c>
       <c r="E14">
         <v>999999</v>
@@ -10825,10 +10818,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C15">
-        <v>18988.505007223368</v>
+        <v>22976.091058740265</v>
       </c>
       <c r="D15">
-        <v>29532.863049035179</v>
+        <v>29532.863049035175</v>
       </c>
       <c r="E15">
         <v>999999</v>
@@ -10842,10 +10835,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C16">
-        <v>18988.505007223368</v>
+        <v>25273.700164614293</v>
       </c>
       <c r="D16">
-        <v>29532.863049035179</v>
+        <v>29532.863049035175</v>
       </c>
       <c r="E16">
         <v>999999</v>
@@ -10859,10 +10852,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C17">
-        <v>18988.505007223368</v>
+        <v>27801.070181075727</v>
       </c>
       <c r="D17">
-        <v>29532.863049035179</v>
+        <v>29532.863049035175</v>
       </c>
       <c r="E17">
         <v>999999</v>
@@ -10876,10 +10869,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C18">
-        <v>18988.505007223368</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="D18">
-        <v>29532.863049035179</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="E18">
         <v>999999</v>
@@ -10893,10 +10886,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C19">
-        <v>18988.505007223368</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="D19">
-        <v>29532.863049035179</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="E19">
         <v>999999</v>
@@ -10910,10 +10903,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C20">
-        <v>18988.505007223368</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="D20">
-        <v>29532.863049035179</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="E20">
         <v>999999</v>
@@ -10927,10 +10920,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C21">
-        <v>18988.505007223368</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="D21">
-        <v>29532.863049035179</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="E21">
         <v>999999</v>
@@ -10944,10 +10937,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C22">
-        <v>18988.505007223368</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="D22">
-        <v>29532.863049035179</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="E22">
         <v>999999</v>
@@ -10961,10 +10954,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C23">
-        <v>18988.505007223368</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="D23">
-        <v>29532.863049035179</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="E23">
         <v>999999</v>
@@ -10978,10 +10971,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C24">
-        <v>18988.505007223368</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="D24">
-        <v>29532.863049035179</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="E24">
         <v>999999</v>
@@ -10995,10 +10988,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C25">
-        <v>18988.505007223368</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="D25">
-        <v>29532.863049035179</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="E25">
         <v>999999</v>
@@ -11012,10 +11005,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C26">
-        <v>18988.505007223368</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="D26">
-        <v>29532.863049035179</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="E26">
         <v>999999</v>
@@ -11029,10 +11022,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C27">
-        <v>18988.505007223368</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="D27">
-        <v>29532.863049035179</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="E27">
         <v>999999</v>
@@ -11046,10 +11039,10 @@
         <v>82878.395711488018</v>
       </c>
       <c r="C28">
-        <v>18988.505007223368</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="D28">
-        <v>29532.863049035179</v>
+        <v>30581.177199183301</v>
       </c>
       <c r="E28">
         <v>999999</v>
@@ -11088,16 +11081,16 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2126230105.0000002</v>
+        <v>211011120.00000003</v>
       </c>
       <c r="C2" s="8">
-        <v>13.655394085392276</v>
+        <v>9.61</v>
       </c>
       <c r="D2">
-        <v>4.9157999999999993E-2</v>
+        <v>6.9372000000000003E-2</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -11105,16 +11098,16 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1477077840.0000002</v>
+        <v>2126230105.0000002</v>
       </c>
       <c r="C3" s="8">
-        <v>34.405314753080312</v>
+        <v>13.66</v>
       </c>
       <c r="D3">
-        <v>3.9239999999999997E-2</v>
+        <v>4.9157999999999993E-2</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -11122,16 +11115,16 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>2321122320</v>
+        <v>81239281.200000003</v>
       </c>
       <c r="C4" s="8">
-        <v>23.606566326931016</v>
+        <v>15.66</v>
       </c>
       <c r="D4">
-        <v>0.19746</v>
+        <v>4.4639999999999999E-2</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -11139,16 +11132,16 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>453673908.00000006</v>
+        <v>167331818.16000003</v>
       </c>
       <c r="C5" s="8">
-        <v>27.373571591866817</v>
+        <v>17.489999999999998</v>
       </c>
       <c r="D5">
-        <v>5.7239999999999999E-2</v>
+        <v>4.4639999999999999E-2</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -11156,16 +11149,16 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>179359452.00000003</v>
+        <v>90734781.600000009</v>
       </c>
       <c r="C6" s="8">
-        <v>20.090694746324271</v>
+        <v>18.18</v>
       </c>
       <c r="D6">
-        <v>4.0806000000000002E-2</v>
+        <v>4.6440000000000002E-2</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -11173,16 +11166,16 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>211011120.00000003</v>
+        <v>1055055600.0000001</v>
       </c>
       <c r="C7" s="8">
-        <v>9.6058634255862909</v>
+        <v>18.87</v>
       </c>
       <c r="D7">
-        <v>6.9372000000000003E-2</v>
+        <v>4.4639999999999999E-2</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -11190,16 +11183,16 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>397755961.20000005</v>
+        <v>179359452.00000003</v>
       </c>
       <c r="C8" s="8">
-        <v>27.656096986737001</v>
+        <v>20.09</v>
       </c>
       <c r="D8">
-        <v>5.7239999999999999E-2</v>
+        <v>4.0806000000000002E-2</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -11207,16 +11200,16 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>167331818.16000003</v>
+        <v>2321122320</v>
       </c>
       <c r="C9" s="8">
-        <v>17.48518277141034</v>
+        <v>23.61</v>
       </c>
       <c r="D9">
-        <v>4.4639999999999999E-2</v>
+        <v>0.19746</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -11224,16 +11217,16 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>220506620.40000001</v>
+        <v>633033360</v>
       </c>
       <c r="C10" s="8">
-        <v>34.405314753080312</v>
+        <v>25.71</v>
       </c>
       <c r="D10">
-        <v>5.7239999999999999E-2</v>
+        <v>5.1839999999999997E-2</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -11241,16 +11234,16 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>90734781.600000009</v>
+        <v>453673908.00000006</v>
       </c>
       <c r="C11" s="8">
-        <v>18.175800403315236</v>
+        <v>27.37</v>
       </c>
       <c r="D11">
-        <v>4.6440000000000002E-2</v>
+        <v>5.7239999999999999E-2</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -11258,16 +11251,16 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>633033360</v>
+        <v>397755961.20000005</v>
       </c>
       <c r="C12" s="8">
-        <v>25.709810933186837</v>
+        <v>27.66</v>
       </c>
       <c r="D12">
-        <v>5.1839999999999997E-2</v>
+        <v>5.7239999999999999E-2</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -11275,16 +11268,16 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>81239281.200000003</v>
+        <v>1477077840.0000002</v>
       </c>
       <c r="C13" s="8">
-        <v>15.664463560024705</v>
+        <v>34.409999999999997</v>
       </c>
       <c r="D13">
-        <v>4.4639999999999999E-2</v>
+        <v>3.9239999999999997E-2</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -11292,16 +11285,16 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>1055055600.0000001</v>
+        <v>220506620.40000001</v>
       </c>
       <c r="C14" s="8">
-        <v>18.866418035220136</v>
+        <v>34.409999999999997</v>
       </c>
       <c r="D14">
-        <v>4.4639999999999999E-2</v>
+        <v>5.7239999999999999E-2</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Fuel prices are not working - CONFIRMED with Excel.
look into the problem, it just does not make any sense how its calculated
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{242CF2B7-D5E0-4759-9FC3-53FB16E4A55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26DF181-503A-4DDD-9E5E-B3E89E525DCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="-5565" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -11202,7 +11202,7 @@
       <c r="B9">
         <v>2321122320</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="8">
         <v>23.61</v>
       </c>
       <c r="D9">
@@ -11219,7 +11219,7 @@
       <c r="B10">
         <v>633033360</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="8">
         <v>25.71</v>
       </c>
       <c r="D10">
@@ -11236,7 +11236,7 @@
       <c r="B11">
         <v>453673908.00000006</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="8">
         <v>27.37</v>
       </c>
       <c r="D11">
@@ -11253,7 +11253,7 @@
       <c r="B12">
         <v>397755961.20000005</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="8">
         <v>27.66</v>
       </c>
       <c r="D12">
@@ -11270,7 +11270,7 @@
       <c r="B13">
         <v>1477077840.0000002</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="8">
         <v>34.409999999999997</v>
       </c>
       <c r="D13">
@@ -11287,7 +11287,7 @@
       <c r="B14">
         <v>220506620.40000001</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="8">
         <v>34.409999999999997</v>
       </c>
       <c r="D14">
@@ -11304,7 +11304,7 @@
       <c r="B15">
         <v>99999999999</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="8">
         <v>1000</v>
       </c>
       <c r="D15">

</xml_diff>

<commit_message>
added O&M Costs resulting in WIth NZIA higher LNG Demand!! Finally
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26DF181-503A-4DDD-9E5E-B3E89E525DCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B802C3-58CC-41DB-9A14-CDBF4AD62AEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="136">
   <si>
     <t>Value</t>
   </si>
@@ -443,6 +443,18 @@
   </si>
   <si>
     <t>Other ME</t>
+  </si>
+  <si>
+    <t>oandm_EU27_solarPV</t>
+  </si>
+  <si>
+    <t>oandm_EU27_windoff</t>
+  </si>
+  <si>
+    <t>oandm_EU27_windon</t>
+  </si>
+  <si>
+    <t>oandm_EU27_Batteries</t>
   </si>
 </sst>
 </file>
@@ -1023,26 +1035,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6185AF38-42FD-4CFF-B287-2FCFFF6C6EF3}">
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:U28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.6640625" customWidth="1"/>
     <col min="3" max="3" width="26.6640625" customWidth="1"/>
-    <col min="4" max="4" width="37.33203125" customWidth="1"/>
-    <col min="5" max="5" width="29.88671875" customWidth="1"/>
-    <col min="6" max="6" width="39.88671875" customWidth="1"/>
-    <col min="7" max="7" width="21.44140625" customWidth="1"/>
-    <col min="9" max="9" width="22.5546875" customWidth="1"/>
-    <col min="10" max="10" width="24.109375" customWidth="1"/>
-    <col min="11" max="11" width="27.6640625" customWidth="1"/>
-    <col min="12" max="12" width="22.88671875" customWidth="1"/>
-    <col min="13" max="13" width="20.109375" customWidth="1"/>
-    <col min="15" max="15" width="32.6640625" customWidth="1"/>
-    <col min="16" max="16" width="35.33203125" customWidth="1"/>
-    <col min="17" max="17" width="31.44140625" customWidth="1"/>
+    <col min="4" max="5" width="37.33203125" customWidth="1"/>
+    <col min="6" max="6" width="29.88671875" customWidth="1"/>
+    <col min="7" max="7" width="39.88671875" customWidth="1"/>
+    <col min="8" max="8" width="21.44140625" customWidth="1"/>
+    <col min="10" max="11" width="22.5546875" customWidth="1"/>
+    <col min="12" max="12" width="24.109375" customWidth="1"/>
+    <col min="13" max="13" width="27.6640625" customWidth="1"/>
+    <col min="14" max="14" width="22.88671875" customWidth="1"/>
+    <col min="15" max="16" width="20.109375" customWidth="1"/>
+    <col min="18" max="18" width="32.6640625" customWidth="1"/>
+    <col min="19" max="19" width="35.33203125" customWidth="1"/>
+    <col min="20" max="20" width="31.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1059,43 +1071,55 @@
         <v>37</v>
       </c>
       <c r="F1" t="s">
+        <v>132</v>
+      </c>
+      <c r="G1" t="s">
         <v>28</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>29</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>30</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>38</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
+        <v>133</v>
+      </c>
+      <c r="L1" t="s">
         <v>43</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>44</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>45</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>46</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q1" t="s">
         <v>52</v>
       </c>
-      <c r="O1" t="s">
+      <c r="R1" t="s">
         <v>53</v>
       </c>
-      <c r="P1" t="s">
+      <c r="S1" t="s">
         <v>54</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="T1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -1112,43 +1136,55 @@
         <v>1000</v>
       </c>
       <c r="F2" s="8">
+        <v>4400</v>
+      </c>
+      <c r="G2" s="8">
         <v>1775265.6417320003</v>
       </c>
-      <c r="G2" s="8">
+      <c r="H2" s="8">
         <v>2337972.5216000001</v>
       </c>
-      <c r="H2" s="8">
+      <c r="I2" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I2" s="8">
+      <c r="J2" s="8">
         <v>1000</v>
       </c>
-      <c r="J2" s="8">
+      <c r="K2" s="8">
+        <v>44000</v>
+      </c>
+      <c r="L2" s="8">
         <v>1052044.8400000001</v>
       </c>
-      <c r="K2" s="8">
+      <c r="M2" s="8">
         <v>1673707.7</v>
       </c>
-      <c r="L2" s="8">
+      <c r="N2" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M2">
+      <c r="O2">
         <v>1000</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="P2">
+        <v>17386.633918245541</v>
+      </c>
+      <c r="Q2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="P2" s="8">
+      <c r="S2" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q2">
+      <c r="T2">
         <v>1000</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -1165,43 +1201,55 @@
         <v>1000</v>
       </c>
       <c r="F3" s="8">
+        <v>4400</v>
+      </c>
+      <c r="G3" s="8">
         <v>1722922.372057667</v>
       </c>
-      <c r="G3" s="8">
+      <c r="H3" s="8">
         <v>2318026.381866667</v>
       </c>
-      <c r="H3" s="8">
+      <c r="I3" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I3" s="8">
+      <c r="J3" s="8">
         <v>1000</v>
       </c>
-      <c r="J3" s="8">
+      <c r="K3" s="8">
+        <v>44000</v>
+      </c>
+      <c r="L3" s="8">
         <v>1042480.7960000001</v>
       </c>
-      <c r="K3" s="8">
+      <c r="M3" s="8">
         <v>1660955.6413333334</v>
       </c>
-      <c r="L3" s="8">
+      <c r="N3" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M3">
+      <c r="O3">
         <v>1000</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="P3">
+        <v>17386.633918245541</v>
+      </c>
+      <c r="Q3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="R3" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="P3" s="8">
+      <c r="S3" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q3">
+      <c r="T3">
         <v>1000</v>
       </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -1218,43 +1266,55 @@
         <v>1000</v>
       </c>
       <c r="F4" s="8">
+        <v>4400</v>
+      </c>
+      <c r="G4" s="8">
         <v>1670579.1023833335</v>
       </c>
-      <c r="G4" s="8">
+      <c r="H4" s="8">
         <v>2298080.2421333333</v>
       </c>
-      <c r="H4" s="8">
+      <c r="I4" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I4" s="8">
+      <c r="J4" s="8">
         <v>1000</v>
       </c>
-      <c r="J4" s="8">
+      <c r="K4" s="8">
+        <v>44000</v>
+      </c>
+      <c r="L4" s="8">
         <v>1032916.7520000001</v>
       </c>
-      <c r="K4" s="8">
+      <c r="M4" s="8">
         <v>1648203.5826666667</v>
       </c>
-      <c r="L4" s="8">
+      <c r="N4" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M4">
+      <c r="O4">
         <v>1000</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="P4">
+        <v>17386.633918245541</v>
+      </c>
+      <c r="Q4" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="P4" s="8">
+      <c r="S4" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q4">
+      <c r="T4">
         <v>1000</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2027</v>
       </c>
@@ -1271,43 +1331,55 @@
         <v>1000</v>
       </c>
       <c r="F5" s="8">
+        <v>4400</v>
+      </c>
+      <c r="G5" s="8">
         <v>1618235.832709</v>
       </c>
-      <c r="G5" s="8">
+      <c r="H5" s="8">
         <v>2278134.1023999997</v>
       </c>
-      <c r="H5" s="8">
+      <c r="I5" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I5" s="8">
+      <c r="J5" s="8">
         <v>1000</v>
       </c>
-      <c r="J5" s="8">
+      <c r="K5" s="8">
+        <v>44000</v>
+      </c>
+      <c r="L5" s="8">
         <v>1023352.708</v>
       </c>
-      <c r="K5" s="8">
+      <c r="M5" s="8">
         <v>1635451.524</v>
       </c>
-      <c r="L5" s="8">
+      <c r="N5" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M5">
+      <c r="O5">
         <v>1000</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="P5">
+        <v>17386.633918245541</v>
+      </c>
+      <c r="Q5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="O5" s="2" t="s">
+      <c r="R5" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="P5" s="8">
+      <c r="S5" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q5">
+      <c r="T5">
         <v>1000</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2028</v>
       </c>
@@ -1324,43 +1396,55 @@
         <v>1000</v>
       </c>
       <c r="F6" s="8">
+        <v>4400</v>
+      </c>
+      <c r="G6" s="8">
         <v>1565892.5630346665</v>
       </c>
-      <c r="G6" s="8">
+      <c r="H6" s="8">
         <v>2258187.9626666661</v>
       </c>
-      <c r="H6" s="8">
+      <c r="I6" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I6" s="8">
+      <c r="J6" s="8">
         <v>1000</v>
       </c>
-      <c r="J6" s="8">
+      <c r="K6" s="8">
+        <v>44000</v>
+      </c>
+      <c r="L6" s="8">
         <v>1013788.6639999999</v>
       </c>
-      <c r="K6" s="8">
+      <c r="M6" s="8">
         <v>1622699.4653333335</v>
       </c>
-      <c r="L6" s="8">
+      <c r="N6" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M6">
+      <c r="O6">
         <v>1000</v>
       </c>
-      <c r="N6" s="2" t="s">
+      <c r="P6">
+        <v>17386.633918245541</v>
+      </c>
+      <c r="Q6" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="O6" s="2" t="s">
+      <c r="R6" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="P6" s="8">
+      <c r="S6" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q6">
+      <c r="T6">
         <v>1000</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2029</v>
       </c>
@@ -1377,43 +1461,55 @@
         <v>1000</v>
       </c>
       <c r="F7" s="8">
+        <v>4400</v>
+      </c>
+      <c r="G7" s="8">
         <v>1513549.293360333</v>
       </c>
-      <c r="G7" s="8">
+      <c r="H7" s="8">
         <v>2238241.8229333302</v>
       </c>
-      <c r="H7" s="8">
+      <c r="I7" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I7" s="8">
+      <c r="J7" s="8">
         <v>1000</v>
       </c>
-      <c r="J7" s="8">
+      <c r="K7" s="8">
+        <v>44000</v>
+      </c>
+      <c r="L7" s="8">
         <v>1004224.62</v>
       </c>
-      <c r="K7" s="8">
+      <c r="M7" s="8">
         <v>1609947.4066666667</v>
       </c>
-      <c r="L7" s="8">
+      <c r="N7" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M7">
+      <c r="O7">
         <v>1000</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="P7">
+        <v>17386.633918245541</v>
+      </c>
+      <c r="Q7" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="O7" s="2" t="s">
+      <c r="R7" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="P7" s="8">
+      <c r="S7" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q7">
+      <c r="T7">
         <v>1000</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -1430,43 +1526,55 @@
         <v>1000</v>
       </c>
       <c r="F8" s="8">
+        <v>3900</v>
+      </c>
+      <c r="G8" s="8">
         <v>1461206.0236859999</v>
       </c>
-      <c r="G8" s="8">
+      <c r="H8" s="8">
         <v>2218295.6831999999</v>
       </c>
-      <c r="H8" s="8">
+      <c r="I8" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I8" s="8">
+      <c r="J8" s="8">
         <v>1000</v>
       </c>
-      <c r="J8" s="8">
+      <c r="K8" s="8">
+        <v>34000</v>
+      </c>
+      <c r="L8" s="8">
         <v>994660.57600000012</v>
       </c>
-      <c r="K8" s="8">
+      <c r="M8" s="8">
         <v>1597195.3480000002</v>
       </c>
-      <c r="L8" s="8">
+      <c r="N8" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M8">
+      <c r="O8">
         <v>1000</v>
       </c>
-      <c r="N8" s="2" t="s">
+      <c r="P8">
+        <v>16662.667964091612</v>
+      </c>
+      <c r="Q8" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="O8" s="2" t="s">
+      <c r="R8" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="P8" s="8">
+      <c r="S8" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q8">
+      <c r="T8">
         <v>1000</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2031</v>
       </c>
@@ -1483,43 +1591,55 @@
         <v>1000</v>
       </c>
       <c r="F9" s="8">
+        <v>3900</v>
+      </c>
+      <c r="G9" s="8">
         <v>1444015.15599508</v>
       </c>
-      <c r="G9" s="8">
+      <c r="H9" s="8">
         <v>2205259.4561600001</v>
       </c>
-      <c r="H9" s="8">
+      <c r="I9" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I9" s="8">
+      <c r="J9" s="8">
         <v>1000</v>
       </c>
-      <c r="J9" s="8">
+      <c r="K9" s="8">
+        <v>34000</v>
+      </c>
+      <c r="L9" s="8">
         <v>992747.76720000012</v>
       </c>
-      <c r="K9" s="8">
+      <c r="M9" s="8">
         <v>1594326.1348000003</v>
       </c>
-      <c r="L9" s="8">
+      <c r="N9" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M9">
+      <c r="O9">
         <v>1000</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="P9">
+        <v>16662.667964091612</v>
+      </c>
+      <c r="Q9" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="O9" s="2" t="s">
+      <c r="R9" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="P9" s="8">
+      <c r="S9" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q9">
+      <c r="T9">
         <v>1000</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2032</v>
       </c>
@@ -1536,43 +1656,55 @@
         <v>1000</v>
       </c>
       <c r="F10" s="8">
+        <v>3900</v>
+      </c>
+      <c r="G10" s="8">
         <v>1426824.2883041599</v>
       </c>
-      <c r="G10" s="8">
+      <c r="H10" s="8">
         <v>2192223.2291199998</v>
       </c>
-      <c r="H10" s="8">
+      <c r="I10" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I10" s="8">
+      <c r="J10" s="8">
         <v>1000</v>
       </c>
-      <c r="J10" s="8">
+      <c r="K10" s="8">
+        <v>34000</v>
+      </c>
+      <c r="L10" s="8">
         <v>990834.9584</v>
       </c>
-      <c r="K10" s="8">
+      <c r="M10" s="8">
         <v>1591456.9216000002</v>
       </c>
-      <c r="L10" s="8">
+      <c r="N10" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M10">
+      <c r="O10">
         <v>1000</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="P10">
+        <v>16662.667964091612</v>
+      </c>
+      <c r="Q10" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="R10" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="P10" s="8">
+      <c r="S10" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q10">
+      <c r="T10">
         <v>1000</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2033</v>
       </c>
@@ -1589,43 +1721,55 @@
         <v>1000</v>
       </c>
       <c r="F11" s="8">
+        <v>3900</v>
+      </c>
+      <c r="G11" s="8">
         <v>1409633.42061324</v>
       </c>
-      <c r="G11" s="8">
+      <c r="H11" s="8">
         <v>2179187.0020799995</v>
       </c>
-      <c r="H11" s="8">
+      <c r="I11" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I11" s="8">
+      <c r="J11" s="8">
         <v>1000</v>
       </c>
-      <c r="J11" s="8">
+      <c r="K11" s="8">
+        <v>34000</v>
+      </c>
+      <c r="L11" s="8">
         <v>988922.1496</v>
       </c>
-      <c r="K11" s="8">
+      <c r="M11" s="8">
         <v>1588587.7084000004</v>
       </c>
-      <c r="L11" s="8">
+      <c r="N11" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M11">
+      <c r="O11">
         <v>1000</v>
       </c>
-      <c r="N11" s="2" t="s">
+      <c r="P11">
+        <v>16662.667964091612</v>
+      </c>
+      <c r="Q11" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="O11" s="2" t="s">
+      <c r="R11" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="P11" s="8">
+      <c r="S11" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q11">
+      <c r="T11">
         <v>1000</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2034</v>
       </c>
@@ -1642,43 +1786,55 @@
         <v>1000</v>
       </c>
       <c r="F12" s="8">
+        <v>3900</v>
+      </c>
+      <c r="G12" s="8">
         <v>1392442.5529223196</v>
       </c>
-      <c r="G12" s="8">
+      <c r="H12" s="8">
         <v>2166150.7750399997</v>
       </c>
-      <c r="H12" s="8">
+      <c r="I12" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I12" s="8">
+      <c r="J12" s="8">
         <v>1000</v>
       </c>
-      <c r="J12" s="8">
+      <c r="K12" s="8">
+        <v>34000</v>
+      </c>
+      <c r="L12" s="8">
         <v>987009.34079999989</v>
       </c>
-      <c r="K12" s="8">
+      <c r="M12" s="8">
         <v>1585718.4952000002</v>
       </c>
-      <c r="L12" s="8">
+      <c r="N12" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M12">
+      <c r="O12">
         <v>1000</v>
       </c>
-      <c r="N12" s="2" t="s">
+      <c r="P12">
+        <v>16662.667964091612</v>
+      </c>
+      <c r="Q12" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="O12" s="2" t="s">
+      <c r="R12" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="P12" s="8">
+      <c r="S12" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q12">
+      <c r="T12">
         <v>1000</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2035</v>
       </c>
@@ -1695,43 +1851,55 @@
         <v>1000</v>
       </c>
       <c r="F13" s="8">
+        <v>3900</v>
+      </c>
+      <c r="G13" s="8">
         <v>1375251.6852313997</v>
       </c>
-      <c r="G13" s="8">
+      <c r="H13" s="8">
         <v>2153114.5479999995</v>
       </c>
-      <c r="H13" s="8">
+      <c r="I13" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I13" s="8">
+      <c r="J13" s="8">
         <v>1000</v>
       </c>
-      <c r="J13" s="8">
+      <c r="K13" s="8">
+        <v>34000</v>
+      </c>
+      <c r="L13" s="8">
         <v>985096.53199999989</v>
       </c>
-      <c r="K13" s="8">
+      <c r="M13" s="8">
         <v>1582849.2820000004</v>
       </c>
-      <c r="L13" s="8">
+      <c r="N13" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M13">
+      <c r="O13">
         <v>1000</v>
       </c>
-      <c r="N13" s="2" t="s">
+      <c r="P13">
+        <v>16662.667964091612</v>
+      </c>
+      <c r="Q13" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="O13" s="2" t="s">
+      <c r="R13" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="P13" s="8">
+      <c r="S13" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q13">
+      <c r="T13">
         <v>1000</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2036</v>
       </c>
@@ -1748,43 +1916,55 @@
         <v>1000</v>
       </c>
       <c r="F14" s="8">
+        <v>3900</v>
+      </c>
+      <c r="G14" s="8">
         <v>1358060.8175404796</v>
       </c>
-      <c r="G14" s="8">
+      <c r="H14" s="8">
         <v>2140078.3209599997</v>
       </c>
-      <c r="H14" s="8">
+      <c r="I14" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I14" s="8">
+      <c r="J14" s="8">
         <v>1000</v>
       </c>
-      <c r="J14" s="8">
+      <c r="K14" s="8">
+        <v>34000</v>
+      </c>
+      <c r="L14" s="8">
         <v>983183.72319999977</v>
       </c>
-      <c r="K14" s="8">
+      <c r="M14" s="8">
         <v>1579980.0688000005</v>
       </c>
-      <c r="L14" s="8">
+      <c r="N14" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M14">
+      <c r="O14">
         <v>1000</v>
       </c>
-      <c r="N14" s="2" t="s">
+      <c r="P14">
+        <v>16662.667964091612</v>
+      </c>
+      <c r="Q14" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="O14" s="2" t="s">
+      <c r="R14" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="P14" s="8">
+      <c r="S14" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q14">
+      <c r="T14">
         <v>1000</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2037</v>
       </c>
@@ -1801,43 +1981,55 @@
         <v>1000</v>
       </c>
       <c r="F15" s="8">
+        <v>3900</v>
+      </c>
+      <c r="G15" s="8">
         <v>1340869.9498495597</v>
       </c>
-      <c r="G15" s="8">
+      <c r="H15" s="8">
         <v>2127042.0939199994</v>
       </c>
-      <c r="H15" s="8">
+      <c r="I15" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I15" s="8">
+      <c r="J15" s="8">
         <v>1000</v>
       </c>
-      <c r="J15" s="8">
+      <c r="K15" s="8">
+        <v>34000</v>
+      </c>
+      <c r="L15" s="8">
         <v>981270.91439999978</v>
       </c>
-      <c r="K15" s="8">
+      <c r="M15" s="8">
         <v>1577110.8556000004</v>
       </c>
-      <c r="L15" s="8">
+      <c r="N15" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M15">
+      <c r="O15">
         <v>1000</v>
       </c>
-      <c r="N15" s="2" t="s">
+      <c r="P15">
+        <v>16662.667964091612</v>
+      </c>
+      <c r="Q15" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="O15" s="2" t="s">
+      <c r="R15" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="P15" s="8">
+      <c r="S15" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q15">
+      <c r="T15">
         <v>1000</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2038</v>
       </c>
@@ -1854,43 +2046,55 @@
         <v>1000</v>
       </c>
       <c r="F16" s="8">
+        <v>3900</v>
+      </c>
+      <c r="G16" s="8">
         <v>1323679.0821586396</v>
       </c>
-      <c r="G16" s="8">
+      <c r="H16" s="8">
         <v>2114005.8668799992</v>
       </c>
-      <c r="H16" s="8">
+      <c r="I16" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I16" s="8">
+      <c r="J16" s="8">
         <v>1000</v>
       </c>
-      <c r="J16" s="8">
+      <c r="K16" s="8">
+        <v>34000</v>
+      </c>
+      <c r="L16" s="8">
         <v>979358.10559999966</v>
       </c>
-      <c r="K16" s="8">
+      <c r="M16" s="8">
         <v>1574241.6424000005</v>
       </c>
-      <c r="L16" s="8">
+      <c r="N16" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M16">
+      <c r="O16">
         <v>1000</v>
       </c>
-      <c r="N16" s="2" t="s">
+      <c r="P16">
+        <v>16662.667964091612</v>
+      </c>
+      <c r="Q16" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="O16" s="2" t="s">
+      <c r="R16" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="P16" s="8">
+      <c r="S16" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q16">
+      <c r="T16">
         <v>1000</v>
       </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2039</v>
       </c>
@@ -1907,43 +2111,55 @@
         <v>1000</v>
       </c>
       <c r="F17" s="8">
+        <v>3900</v>
+      </c>
+      <c r="G17" s="8">
         <v>1306488.2144677194</v>
       </c>
-      <c r="G17" s="8">
+      <c r="H17" s="8">
         <v>2100969.6398399994</v>
       </c>
-      <c r="H17" s="8">
+      <c r="I17" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I17" s="8">
+      <c r="J17" s="8">
         <v>1000</v>
       </c>
-      <c r="J17" s="8">
+      <c r="K17" s="8">
+        <v>34000</v>
+      </c>
+      <c r="L17" s="8">
         <v>977445.29679999966</v>
       </c>
-      <c r="K17" s="8">
+      <c r="M17" s="8">
         <v>1571372.4292000004</v>
       </c>
-      <c r="L17" s="8">
+      <c r="N17" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M17">
+      <c r="O17">
         <v>1000</v>
       </c>
-      <c r="N17" s="2" t="s">
+      <c r="P17">
+        <v>16662.667964091612</v>
+      </c>
+      <c r="Q17" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="O17" s="2" t="s">
+      <c r="R17" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="P17" s="8">
+      <c r="S17" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q17">
+      <c r="T17">
         <v>1000</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2040</v>
       </c>
@@ -1960,43 +2176,55 @@
         <v>1000</v>
       </c>
       <c r="F18" s="8">
+        <v>3100</v>
+      </c>
+      <c r="G18" s="8">
         <v>1288027.7959324</v>
       </c>
-      <c r="G18" s="8">
+      <c r="H18" s="8">
         <v>2087933.4128</v>
       </c>
-      <c r="H18" s="8">
+      <c r="I18" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I18" s="8">
+      <c r="J18" s="8">
         <v>1000</v>
       </c>
-      <c r="J18" s="8">
+      <c r="K18" s="8">
+        <v>30000</v>
+      </c>
+      <c r="L18" s="8">
         <v>975532.48799999955</v>
       </c>
-      <c r="K18" s="8">
+      <c r="M18" s="8">
         <v>1568503.2160000005</v>
       </c>
-      <c r="L18" s="8">
+      <c r="N18" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M18">
+      <c r="O18">
         <v>1000</v>
       </c>
-      <c r="N18" s="2" t="s">
+      <c r="P18">
+        <v>15965.364846295015</v>
+      </c>
+      <c r="Q18" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="O18" s="2" t="s">
+      <c r="R18" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="P18" s="8">
+      <c r="S18" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q18">
+      <c r="T18">
         <v>1000</v>
       </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2041</v>
       </c>
@@ -2013,43 +2241,55 @@
         <v>1000</v>
       </c>
       <c r="F19" s="8">
+        <v>3100</v>
+      </c>
+      <c r="G19" s="8">
         <v>1288154.7510168403</v>
       </c>
-      <c r="G19" s="8">
+      <c r="H19" s="8">
         <v>2076927.41784</v>
       </c>
-      <c r="H19" s="8">
+      <c r="I19" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I19" s="8">
+      <c r="J19" s="8">
         <v>1000</v>
       </c>
-      <c r="J19" s="8">
+      <c r="K19" s="8">
+        <v>30000</v>
+      </c>
+      <c r="L19" s="8">
         <v>973619.67919999966</v>
       </c>
-      <c r="K19" s="8">
+      <c r="M19" s="8">
         <v>1565634.0028000006</v>
       </c>
-      <c r="L19" s="8">
+      <c r="N19" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M19">
+      <c r="O19">
         <v>1000</v>
       </c>
-      <c r="N19" s="2" t="s">
+      <c r="P19">
+        <v>15965.364846295015</v>
+      </c>
+      <c r="Q19" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="O19" s="2" t="s">
+      <c r="R19" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="P19" s="8">
+      <c r="S19" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q19">
+      <c r="T19">
         <v>1000</v>
       </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2042</v>
       </c>
@@ -2066,43 +2306,55 @@
         <v>1000</v>
       </c>
       <c r="F20" s="8">
+        <v>3100</v>
+      </c>
+      <c r="G20" s="8">
         <v>1288281.7061012802</v>
       </c>
-      <c r="G20" s="8">
+      <c r="H20" s="8">
         <v>2065921.4228800002</v>
       </c>
-      <c r="H20" s="8">
+      <c r="I20" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I20" s="8">
+      <c r="J20" s="8">
         <v>1000</v>
       </c>
-      <c r="J20" s="8">
+      <c r="K20" s="8">
+        <v>30000</v>
+      </c>
+      <c r="L20" s="8">
         <v>971706.87039999955</v>
       </c>
-      <c r="K20" s="8">
+      <c r="M20" s="8">
         <v>1562764.7896000005</v>
       </c>
-      <c r="L20" s="8">
+      <c r="N20" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M20">
+      <c r="O20">
         <v>1000</v>
       </c>
-      <c r="N20" s="2" t="s">
+      <c r="P20">
+        <v>15965.364846295015</v>
+      </c>
+      <c r="Q20" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="O20" s="2" t="s">
+      <c r="R20" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="P20" s="8">
+      <c r="S20" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q20">
+      <c r="T20">
         <v>1000</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2043</v>
       </c>
@@ -2119,43 +2371,55 @@
         <v>1000</v>
       </c>
       <c r="F21" s="8">
+        <v>3100</v>
+      </c>
+      <c r="G21" s="8">
         <v>1288408.6611857202</v>
       </c>
-      <c r="G21" s="8">
+      <c r="H21" s="8">
         <v>2054915.4279200002</v>
       </c>
-      <c r="H21" s="8">
+      <c r="I21" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I21" s="8">
+      <c r="J21" s="8">
         <v>1000</v>
       </c>
-      <c r="J21" s="8">
+      <c r="K21" s="8">
+        <v>30000</v>
+      </c>
+      <c r="L21" s="8">
         <v>969794.06159999955</v>
       </c>
-      <c r="K21" s="8">
+      <c r="M21" s="8">
         <v>1559895.5764000006</v>
       </c>
-      <c r="L21" s="8">
+      <c r="N21" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M21">
+      <c r="O21">
         <v>1000</v>
       </c>
-      <c r="N21" s="2" t="s">
+      <c r="P21">
+        <v>15965.364846295015</v>
+      </c>
+      <c r="Q21" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="O21" s="2" t="s">
+      <c r="R21" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="P21" s="8">
+      <c r="S21" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q21">
+      <c r="T21">
         <v>1000</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2044</v>
       </c>
@@ -2172,43 +2436,55 @@
         <v>1000</v>
       </c>
       <c r="F22" s="8">
+        <v>3100</v>
+      </c>
+      <c r="G22" s="8">
         <v>1288535.6162701603</v>
       </c>
-      <c r="G22" s="8">
+      <c r="H22" s="8">
         <v>2043909.4329600004</v>
       </c>
-      <c r="H22" s="8">
+      <c r="I22" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I22" s="8">
+      <c r="J22" s="8">
         <v>1000</v>
       </c>
-      <c r="J22" s="8">
+      <c r="K22" s="8">
+        <v>30000</v>
+      </c>
+      <c r="L22" s="8">
         <v>967881.25279999943</v>
       </c>
-      <c r="K22" s="8">
+      <c r="M22" s="8">
         <v>1557026.3632000005</v>
       </c>
-      <c r="L22" s="8">
+      <c r="N22" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M22">
+      <c r="O22">
         <v>1000</v>
       </c>
-      <c r="N22" s="2" t="s">
+      <c r="P22">
+        <v>15965.364846295015</v>
+      </c>
+      <c r="Q22" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="O22" s="2" t="s">
+      <c r="R22" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="P22" s="8">
+      <c r="S22" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q22">
+      <c r="T22">
         <v>1000</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2045</v>
       </c>
@@ -2225,43 +2501,55 @@
         <v>1000</v>
       </c>
       <c r="F23" s="8">
+        <v>3100</v>
+      </c>
+      <c r="G23" s="8">
         <v>1288662.5713546001</v>
       </c>
-      <c r="G23" s="8">
+      <c r="H23" s="8">
         <v>2032903.4380000005</v>
       </c>
-      <c r="H23" s="8">
+      <c r="I23" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I23" s="8">
+      <c r="J23" s="8">
         <v>1000</v>
       </c>
-      <c r="J23" s="8">
+      <c r="K23" s="8">
+        <v>30000</v>
+      </c>
+      <c r="L23" s="8">
         <v>965968.44399999944</v>
       </c>
-      <c r="K23" s="8">
+      <c r="M23" s="8">
         <v>1554157.1500000006</v>
       </c>
-      <c r="L23" s="8">
+      <c r="N23" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M23">
+      <c r="O23">
         <v>1000</v>
       </c>
-      <c r="N23" s="2" t="s">
+      <c r="P23">
+        <v>15965.364846295015</v>
+      </c>
+      <c r="Q23" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="O23" s="2" t="s">
+      <c r="R23" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="P23" s="8">
+      <c r="S23" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q23">
+      <c r="T23">
         <v>1000</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2046</v>
       </c>
@@ -2278,43 +2566,55 @@
         <v>1000</v>
       </c>
       <c r="F24" s="8">
+        <v>3100</v>
+      </c>
+      <c r="G24" s="8">
         <v>1288789.5264390404</v>
       </c>
-      <c r="G24" s="8">
+      <c r="H24" s="8">
         <v>2021897.4430400007</v>
       </c>
-      <c r="H24" s="8">
+      <c r="I24" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I24" s="8">
+      <c r="J24" s="8">
         <v>1000</v>
       </c>
-      <c r="J24" s="8">
+      <c r="K24" s="8">
+        <v>30000</v>
+      </c>
+      <c r="L24" s="8">
         <v>964055.63519999932</v>
       </c>
-      <c r="K24" s="8">
+      <c r="M24" s="8">
         <v>1551287.9368000007</v>
       </c>
-      <c r="L24" s="8">
+      <c r="N24" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M24">
+      <c r="O24">
         <v>1000</v>
       </c>
-      <c r="N24" s="2" t="s">
+      <c r="P24">
+        <v>15965.364846295015</v>
+      </c>
+      <c r="Q24" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="O24" s="2" t="s">
+      <c r="R24" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="P24" s="8">
+      <c r="S24" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q24">
+      <c r="T24">
         <v>1000</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2047</v>
       </c>
@@ -2331,43 +2631,55 @@
         <v>1000</v>
       </c>
       <c r="F25" s="8">
+        <v>3100</v>
+      </c>
+      <c r="G25" s="8">
         <v>1288916.4815234803</v>
       </c>
-      <c r="G25" s="8">
+      <c r="H25" s="8">
         <v>2010891.4480800009</v>
       </c>
-      <c r="H25" s="8">
+      <c r="I25" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I25" s="8">
+      <c r="J25" s="8">
         <v>1000</v>
       </c>
-      <c r="J25" s="8">
+      <c r="K25" s="8">
+        <v>30000</v>
+      </c>
+      <c r="L25" s="8">
         <v>962142.82639999932</v>
       </c>
-      <c r="K25" s="8">
+      <c r="M25" s="8">
         <v>1548418.7236000006</v>
       </c>
-      <c r="L25" s="8">
+      <c r="N25" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M25">
+      <c r="O25">
         <v>1000</v>
       </c>
-      <c r="N25" s="2" t="s">
+      <c r="P25">
+        <v>15965.364846295015</v>
+      </c>
+      <c r="Q25" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="O25" s="2" t="s">
+      <c r="R25" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="P25" s="8">
+      <c r="S25" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q25">
+      <c r="T25">
         <v>1000</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2048</v>
       </c>
@@ -2384,43 +2696,55 @@
         <v>1000</v>
       </c>
       <c r="F26" s="8">
+        <v>3100</v>
+      </c>
+      <c r="G26" s="8">
         <v>1289043.4366079206</v>
       </c>
-      <c r="G26" s="8">
+      <c r="H26" s="8">
         <v>1999885.4531200009</v>
       </c>
-      <c r="H26" s="8">
+      <c r="I26" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I26" s="8">
+      <c r="J26" s="8">
         <v>1000</v>
       </c>
-      <c r="J26" s="8">
+      <c r="K26" s="8">
+        <v>30000</v>
+      </c>
+      <c r="L26" s="8">
         <v>960230.01759999921</v>
       </c>
-      <c r="K26" s="8">
+      <c r="M26" s="8">
         <v>1545549.5104000007</v>
       </c>
-      <c r="L26" s="8">
+      <c r="N26" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M26">
+      <c r="O26">
         <v>1000</v>
       </c>
-      <c r="N26" s="2" t="s">
+      <c r="P26">
+        <v>15965.364846295015</v>
+      </c>
+      <c r="Q26" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="O26" s="2" t="s">
+      <c r="R26" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="P26" s="8">
+      <c r="S26" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q26">
+      <c r="T26">
         <v>1000</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2049</v>
       </c>
@@ -2437,43 +2761,55 @@
         <v>1000</v>
       </c>
       <c r="F27" s="8">
+        <v>3100</v>
+      </c>
+      <c r="G27" s="8">
         <v>1289170.3916923604</v>
       </c>
-      <c r="G27" s="8">
+      <c r="H27" s="8">
         <v>1988879.4581600011</v>
       </c>
-      <c r="H27" s="8">
+      <c r="I27" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I27" s="8">
+      <c r="J27" s="8">
         <v>1000</v>
       </c>
-      <c r="J27" s="8">
+      <c r="K27" s="8">
+        <v>30000</v>
+      </c>
+      <c r="L27" s="8">
         <v>958317.20879999921</v>
       </c>
-      <c r="K27" s="8">
+      <c r="M27" s="8">
         <v>1542680.2972000006</v>
       </c>
-      <c r="L27" s="8">
+      <c r="N27" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M27">
+      <c r="O27">
         <v>1000</v>
       </c>
-      <c r="N27" s="2" t="s">
+      <c r="P27">
+        <v>15965.364846295015</v>
+      </c>
+      <c r="Q27" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="O27" s="2" t="s">
+      <c r="R27" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="P27" s="8">
+      <c r="S27" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q27">
+      <c r="T27">
         <v>1000</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="U27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2050</v>
       </c>
@@ -2490,40 +2826,52 @@
         <v>1000</v>
       </c>
       <c r="F28" s="8">
+        <v>2500</v>
+      </c>
+      <c r="G28" s="8">
         <v>1289297.3467768</v>
       </c>
-      <c r="G28" s="8">
+      <c r="H28" s="8">
         <v>1977873.4631999999</v>
       </c>
-      <c r="H28" s="8">
+      <c r="I28" s="8">
         <v>1646946.1610000001</v>
       </c>
-      <c r="I28" s="8">
+      <c r="J28" s="8">
         <v>1000</v>
       </c>
-      <c r="J28" s="8">
+      <c r="K28" s="8">
+        <v>28000</v>
+      </c>
+      <c r="L28" s="8">
         <v>956404.40000000026</v>
       </c>
-      <c r="K28" s="8">
+      <c r="M28" s="8">
         <v>1539811.0840000003</v>
       </c>
-      <c r="L28" s="8">
+      <c r="N28" s="8">
         <v>1093231.041</v>
       </c>
-      <c r="M28">
+      <c r="O28">
         <v>1000</v>
       </c>
-      <c r="N28" s="2" t="s">
+      <c r="P28">
+        <v>15602.06928231802</v>
+      </c>
+      <c r="Q28" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="O28" s="2" t="s">
+      <c r="R28" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="P28" s="8">
+      <c r="S28" s="8">
         <v>489061.86</v>
       </c>
-      <c r="Q28">
+      <c r="T28">
         <v>1000</v>
+      </c>
+      <c r="U28">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implementation of Gas done, TODO:
look at min-fraction value, maybe we can trim Balance Output towards that..  Only question is how fuel input is affected
</commit_message>
<xml_diff>
--- a/Input_urbsextensionv1.xlsx
+++ b/Input_urbsextensionv1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAAB626C-FF8B-49DC-9212-F08D6DF01308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB3966CB-6233-4861-A1AB-524FA1662BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="8" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
+    <workbookView xWindow="67080" yWindow="-5565" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="4" xr2:uid="{81864710-3A67-40FC-ABA1-4EF02E4F8A12}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="10" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <sheet name="gas_block" sheetId="13" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">gas_block!$C$1:$C$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">gas_block!$B$1:$B$109</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -446,7 +446,7 @@
     </xf>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -474,7 +474,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -491,28 +490,7 @@
     <cellStyle name="N_Table1_Header" xfId="6" xr:uid="{5B945886-E1B9-4000-BFBC-F4E856A0CA51}"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -9414,7 +9392,7 @@
         <v>27</v>
       </c>
       <c r="B2" s="11">
-        <v>304000</v>
+        <v>211115</v>
       </c>
       <c r="C2" s="6">
         <v>40000</v>
@@ -9435,7 +9413,7 @@
         <v>0</v>
       </c>
       <c r="I2" s="6">
-        <v>0.37409999999999999</v>
+        <v>0.24030000000000001</v>
       </c>
       <c r="J2" s="6">
         <v>0.38879999999999998</v>
@@ -9512,7 +9490,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="6">
-        <v>7000</v>
+        <v>5000</v>
       </c>
       <c r="H3" s="5">
         <v>0</v>
@@ -9580,7 +9558,7 @@
         <v>41</v>
       </c>
       <c r="B4" s="7">
-        <v>210000</v>
+        <v>195370</v>
       </c>
       <c r="C4" s="7">
         <v>0</v>
@@ -9595,7 +9573,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="6">
-        <v>23000</v>
+        <v>20000</v>
       </c>
       <c r="H4" s="5">
         <v>0</v>
@@ -11254,16 +11232,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="12" t="s">
         <v>62</v>
       </c>
       <c r="G1" s="10" t="s">
@@ -11271,16 +11249,16 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="12">
+      <c r="A2" s="13">
         <v>2024</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D2" s="13">
+      <c r="D2">
         <v>29.19</v>
       </c>
       <c r="G2" s="10">
@@ -11288,14 +11266,14 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="12"/>
-      <c r="B3" s="14" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D3" s="13">
+      <c r="C3" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D3">
         <v>42.69</v>
       </c>
       <c r="G3" s="10">
@@ -11303,14 +11281,14 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="12"/>
-      <c r="B4" s="14" t="s">
+      <c r="A4" s="13"/>
+      <c r="B4" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D4" s="13">
+      <c r="C4" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D4">
         <v>150</v>
       </c>
       <c r="G4" s="10">
@@ -11318,1339 +11296,1320 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="12"/>
-      <c r="B5" s="14" t="s">
+      <c r="A5" s="13"/>
+      <c r="B5" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="13">
-        <v>319200000</v>
-      </c>
-      <c r="D5" s="13">
+      <c r="C5" s="2">
+        <v>532000000</v>
+      </c>
+      <c r="D5">
         <v>22.68</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="12">
+      <c r="A6" s="13">
         <v>2025</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6">
         <v>29.19</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="12"/>
-      <c r="B7" s="14" t="s">
+      <c r="A7" s="13"/>
+      <c r="B7" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D7" s="13">
+      <c r="C7" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D7">
         <v>42.69</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="12"/>
-      <c r="B8" s="14" t="s">
+      <c r="A8" s="13"/>
+      <c r="B8" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D8" s="13">
+      <c r="C8" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D8">
         <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="12"/>
-      <c r="B9" s="14" t="s">
+      <c r="A9" s="13"/>
+      <c r="B9" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="13">
-        <v>306266016</v>
-      </c>
-      <c r="D9" s="13">
+      <c r="C9" s="2">
+        <v>510132160</v>
+      </c>
+      <c r="D9">
         <v>22.545000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="12">
+      <c r="A10" s="13">
         <v>2026</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10">
         <v>29.19</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="12"/>
-      <c r="B11" s="14" t="s">
+      <c r="A11" s="13"/>
+      <c r="B11" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D11" s="13">
+      <c r="C11" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D11">
         <v>42.69</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="12"/>
-      <c r="B12" s="14" t="s">
+      <c r="A12" s="13"/>
+      <c r="B12" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D12" s="13">
+      <c r="C12" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D12">
         <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="12"/>
-      <c r="B13" s="14" t="s">
+      <c r="A13" s="13"/>
+      <c r="B13" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="13">
-        <v>293856117.03167999</v>
-      </c>
-      <c r="D13" s="13">
+      <c r="C13" s="2">
+        <v>489197947</v>
+      </c>
+      <c r="D13">
         <v>22.41</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="12">
+      <c r="A14" s="13">
         <v>2027</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D14">
         <v>29.19</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="12"/>
-      <c r="B15" s="14" t="s">
+      <c r="A15" s="13"/>
+      <c r="B15" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C15" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D15" s="13">
+      <c r="C15" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D15">
         <v>42.69</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="12"/>
-      <c r="B16" s="14" t="s">
+      <c r="A16" s="13"/>
+      <c r="B16" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C16" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D16" s="13">
+      <c r="C16" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D16">
         <v>150</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="12"/>
-      <c r="B17" s="14" t="s">
+      <c r="A17" s="13"/>
+      <c r="B17" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="13">
-        <v>281949067.16955632</v>
-      </c>
-      <c r="D17" s="13">
+      <c r="C17" s="2">
+        <v>469163758</v>
+      </c>
+      <c r="D17">
         <v>22.274999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="12">
+      <c r="A18" s="13">
         <v>2028</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D18" s="13">
+      <c r="D18">
         <v>29.19</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="12"/>
-      <c r="B19" s="14" t="s">
+      <c r="A19" s="13"/>
+      <c r="B19" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C19" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D19" s="13">
+      <c r="C19" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D19">
         <v>42.69</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="12"/>
-      <c r="B20" s="14" t="s">
+      <c r="A20" s="13"/>
+      <c r="B20" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C20" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D20" s="13">
+      <c r="C20" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D20">
         <v>150</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="12"/>
-      <c r="B21" s="14" t="s">
+      <c r="A21" s="13"/>
+      <c r="B21" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="13">
-        <v>270524490.96784592</v>
-      </c>
-      <c r="D21" s="13">
+      <c r="C21" s="2">
+        <v>449997786</v>
+      </c>
+      <c r="D21">
         <v>22.14</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="12">
+      <c r="A22" s="13">
         <v>2029</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="13">
+      <c r="C22" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D22" s="13">
+      <c r="D22">
         <v>29.19</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="12"/>
-      <c r="B23" s="14" t="s">
+      <c r="A23" s="13"/>
+      <c r="B23" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C23" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D23" s="13">
+      <c r="C23" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D23">
         <v>42.69</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="12"/>
-      <c r="B24" s="14" t="s">
+      <c r="A24" s="13"/>
+      <c r="B24" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C24" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D24" s="13">
+      <c r="C24" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D24">
         <v>150</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="12"/>
-      <c r="B25" s="14" t="s">
+      <c r="A25" s="13"/>
+      <c r="B25" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="13">
-        <v>259562838.5938288</v>
-      </c>
-      <c r="D25" s="13">
+      <c r="C25" s="2">
+        <v>431671839</v>
+      </c>
+      <c r="D25">
         <v>22.004999999999999</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="12">
+      <c r="A26" s="13">
         <v>2030</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C26" s="13">
+      <c r="C26" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D26" s="13">
+      <c r="D26">
         <v>29.19</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="12"/>
-      <c r="B27" s="14" t="s">
+      <c r="A27" s="13"/>
+      <c r="B27" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C27" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D27" s="13">
+      <c r="C27" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D27">
         <v>42.69</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="12"/>
-      <c r="B28" s="14" t="s">
+      <c r="A28" s="13"/>
+      <c r="B28" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C28" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D28" s="13">
+      <c r="C28" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D28">
         <v>150</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="12"/>
-      <c r="B29" s="14" t="s">
+      <c r="A29" s="13"/>
+      <c r="B29" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C29" s="13">
-        <v>249045352.37400681</v>
-      </c>
-      <c r="D29" s="13">
+      <c r="C29" s="2">
+        <v>414151522</v>
+      </c>
+      <c r="D29">
         <v>21.87</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="12">
+      <c r="A30" s="13">
         <v>2031</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B30" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="13">
+      <c r="C30" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D30" s="13">
+      <c r="D30">
         <v>29.19</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="12"/>
-      <c r="B31" s="14" t="s">
+      <c r="A31" s="13"/>
+      <c r="B31" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C31" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D31" s="13">
+      <c r="C31" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D31">
         <v>42.69</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="12"/>
-      <c r="B32" s="14" t="s">
+      <c r="A32" s="13"/>
+      <c r="B32" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C32" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D32" s="13">
+      <c r="C32" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D32">
         <v>150</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="12"/>
-      <c r="B33" s="14" t="s">
+      <c r="A33" s="13"/>
+      <c r="B33" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C33" s="13">
-        <v>238954034.69581211</v>
-      </c>
-      <c r="D33" s="13">
+      <c r="C33" s="2">
+        <v>397404638</v>
+      </c>
+      <c r="D33">
         <v>21.734999999999999</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="12">
+      <c r="A34" s="13">
         <v>2032</v>
       </c>
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C34" s="13">
+      <c r="C34" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D34" s="13">
+      <c r="D34">
         <v>29.19</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="12"/>
-      <c r="B35" s="14" t="s">
+      <c r="A35" s="13"/>
+      <c r="B35" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C35" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D35" s="13">
+      <c r="C35" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D35">
         <v>42.69</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="12"/>
-      <c r="B36" s="14" t="s">
+      <c r="A36" s="13"/>
+      <c r="B36" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C36" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D36" s="13">
+      <c r="C36" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D36">
         <v>150</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="12"/>
-      <c r="B37" s="14" t="s">
+      <c r="A37" s="13"/>
+      <c r="B37" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C37" s="13">
-        <v>229271617.20993781</v>
-      </c>
-      <c r="D37" s="13">
+      <c r="C37" s="2">
+        <v>381406956</v>
+      </c>
+      <c r="D37">
         <v>21.6</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="12">
+      <c r="A38" s="13">
         <v>2033</v>
       </c>
-      <c r="B38" s="14" t="s">
+      <c r="B38" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C38" s="13">
+      <c r="C38" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D38" s="13">
+      <c r="D38">
         <v>29.19</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="12"/>
-      <c r="B39" s="14" t="s">
+      <c r="A39" s="13"/>
+      <c r="B39" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C39" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D39" s="13">
+      <c r="C39" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D39">
         <v>42.69</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="12"/>
-      <c r="B40" s="14" t="s">
+      <c r="A40" s="13"/>
+      <c r="B40" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C40" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D40" s="13">
+      <c r="C40" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D40">
         <v>150</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="12"/>
-      <c r="B41" s="14" t="s">
+      <c r="A41" s="13"/>
+      <c r="B41" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C41" s="13">
-        <v>219981531.2805911</v>
-      </c>
-      <c r="D41" s="13">
+      <c r="C41" s="2">
+        <v>366136021</v>
+      </c>
+      <c r="D41">
         <v>21.465</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="12">
+      <c r="A42" s="13">
         <v>2034</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B42" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C42" s="13">
+      <c r="C42" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D42" s="13">
+      <c r="D42">
         <v>29.19</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="12"/>
-      <c r="B43" s="14" t="s">
+      <c r="A43" s="13"/>
+      <c r="B43" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C43" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D43" s="13">
+      <c r="C43" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D43">
         <v>42.69</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="12"/>
-      <c r="B44" s="14" t="s">
+      <c r="A44" s="13"/>
+      <c r="B44" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C44" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D44" s="13">
+      <c r="C44" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D44">
         <v>150</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A45" s="12"/>
-      <c r="B45" s="14" t="s">
+      <c r="A45" s="13"/>
+      <c r="B45" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="13">
-        <v>211067879.63310149</v>
-      </c>
-      <c r="D45" s="13">
+      <c r="C45" s="2">
+        <v>351566712</v>
+      </c>
+      <c r="D45">
         <v>21.33</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46" s="12">
+      <c r="A46" s="13">
         <v>2035</v>
       </c>
-      <c r="B46" s="14" t="s">
+      <c r="B46" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C46" s="13">
+      <c r="C46" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D46" s="13">
+      <c r="D46">
         <v>29.19</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="12"/>
-      <c r="B47" s="14" t="s">
+      <c r="A47" s="13"/>
+      <c r="B47" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C47" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D47" s="13">
+      <c r="C47" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D47">
         <v>42.69</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A48" s="12"/>
-      <c r="B48" s="14" t="s">
+      <c r="A48" s="13"/>
+      <c r="B48" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C48" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D48" s="13">
+      <c r="C48" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D48">
         <v>150</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="12"/>
-      <c r="B49" s="14" t="s">
+      <c r="A49" s="13"/>
+      <c r="B49" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C49" s="13">
-        <v>202515409.1503683</v>
-      </c>
-      <c r="D49" s="13">
+      <c r="C49" s="2">
+        <v>337680248</v>
+      </c>
+      <c r="D49">
         <v>21.195</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A50" s="12">
+      <c r="A50" s="13">
         <v>2036</v>
       </c>
-      <c r="B50" s="14" t="s">
+      <c r="B50" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C50" s="13">
+      <c r="C50" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D50" s="13">
+      <c r="D50">
         <v>29.19</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="12"/>
-      <c r="B51" s="14" t="s">
+      <c r="A51" s="13"/>
+      <c r="B51" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C51" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D51" s="13">
+      <c r="C51" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D51">
         <v>42.69</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A52" s="12"/>
-      <c r="B52" s="14" t="s">
+      <c r="A52" s="13"/>
+      <c r="B52" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C52" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D52" s="13">
+      <c r="C52" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D52">
         <v>150</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" s="12"/>
-      <c r="B53" s="14" t="s">
+      <c r="A53" s="13"/>
+      <c r="B53" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C53" s="13">
-        <v>194309484.77159539</v>
-      </c>
-      <c r="D53" s="13">
+      <c r="C53" s="2">
+        <v>324452734</v>
+      </c>
+      <c r="D53">
         <v>21.06</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="12">
+      <c r="A54" s="13">
         <v>2037</v>
       </c>
-      <c r="B54" s="14" t="s">
+      <c r="B54" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C54" s="13">
+      <c r="C54" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D54" s="13">
+      <c r="D54">
         <v>29.19</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" s="12"/>
-      <c r="B55" s="14" t="s">
+      <c r="A55" s="13"/>
+      <c r="B55" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C55" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D55" s="13">
+      <c r="C55" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D55">
         <v>42.69</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A56" s="12"/>
-      <c r="B56" s="14" t="s">
+      <c r="A56" s="13"/>
+      <c r="B56" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C56" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D56" s="13">
+      <c r="C56" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D56">
         <v>150</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A57" s="12"/>
-      <c r="B57" s="14" t="s">
+      <c r="A57" s="13"/>
+      <c r="B57" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C57" s="13">
-        <v>186436064.4486503</v>
-      </c>
-      <c r="D57" s="13">
+      <c r="C57" s="2">
+        <v>311864566</v>
+      </c>
+      <c r="D57">
         <v>20.925000000000001</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A58" s="12">
+      <c r="A58" s="13">
         <v>2038</v>
       </c>
-      <c r="B58" s="14" t="s">
+      <c r="B58" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C58" s="13">
+      <c r="C58" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D58" s="13">
+      <c r="D58">
         <v>29.19</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" s="12"/>
-      <c r="B59" s="14" t="s">
+      <c r="A59" s="13"/>
+      <c r="B59" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C59" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D59" s="13">
+      <c r="C59" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D59">
         <v>42.69</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A60" s="12"/>
-      <c r="B60" s="14" t="s">
+      <c r="A60" s="13"/>
+      <c r="B60" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C60" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D60" s="13">
+      <c r="C60" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D60">
         <v>150</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A61" s="12"/>
-      <c r="B61" s="14" t="s">
+      <c r="A61" s="13"/>
+      <c r="B61" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C61" s="13">
-        <v>178881675.11719099</v>
-      </c>
-      <c r="D61" s="13">
+      <c r="C61" s="2">
+        <v>299896970</v>
+      </c>
+      <c r="D61">
         <v>20.79</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A62" s="12">
+      <c r="A62" s="13">
         <v>2039</v>
       </c>
-      <c r="B62" s="14" t="s">
+      <c r="B62" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C62" s="13">
+      <c r="C62" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D62" s="13">
+      <c r="D62">
         <v>29.19</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A63" s="12"/>
-      <c r="B63" s="14" t="s">
+      <c r="A63" s="13"/>
+      <c r="B63" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C63" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D63" s="13">
+      <c r="C63" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D63">
         <v>42.69</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A64" s="12"/>
-      <c r="B64" s="14" t="s">
+      <c r="A64" s="13"/>
+      <c r="B64" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C64" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D64" s="13">
+      <c r="C64" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D64">
         <v>150</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" s="12"/>
-      <c r="B65" s="14" t="s">
+      <c r="A65" s="13"/>
+      <c r="B65" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C65" s="13">
-        <v>171633389.64144239</v>
-      </c>
-      <c r="D65" s="13">
+      <c r="C65" s="2">
+        <v>288530884</v>
+      </c>
+      <c r="D65">
         <v>20.655000000000001</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" s="12">
+      <c r="A66" s="13">
         <v>2040</v>
       </c>
-      <c r="B66" s="14" t="s">
+      <c r="B66" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C66" s="13">
+      <c r="C66" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D66" s="13">
+      <c r="D66">
         <v>29.19</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" s="12"/>
-      <c r="B67" s="14" t="s">
+      <c r="A67" s="13"/>
+      <c r="B67" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C67" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D67" s="13">
+      <c r="C67" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D67">
         <v>42.69</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" s="12"/>
-      <c r="B68" s="14" t="s">
+      <c r="A68" s="13"/>
+      <c r="B68" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C68" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D68" s="13">
+      <c r="C68" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D68">
         <v>150</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A69" s="12"/>
-      <c r="B69" s="14" t="s">
+      <c r="A69" s="13"/>
+      <c r="B69" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C69" s="13">
-        <v>164678804.6931712</v>
-      </c>
-      <c r="D69" s="13">
+      <c r="C69" s="2">
+        <v>277748804</v>
+      </c>
+      <c r="D69">
         <v>20.52</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A70" s="12">
+      <c r="A70" s="13">
         <v>2041</v>
       </c>
-      <c r="B70" s="14" t="s">
+      <c r="B70" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C70" s="13">
+      <c r="C70" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D70" s="13">
+      <c r="D70">
         <v>29.19</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A71" s="12"/>
-      <c r="B71" s="14" t="s">
+      <c r="A71" s="13"/>
+      <c r="B71" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C71" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D71" s="13">
+      <c r="C71" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D71">
         <v>42.69</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A72" s="12"/>
-      <c r="B72" s="14" t="s">
+      <c r="A72" s="13"/>
+      <c r="B72" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C72" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D72" s="13">
+      <c r="C72" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D72">
         <v>150</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" s="12"/>
-      <c r="B73" s="14" t="s">
+      <c r="A73" s="13"/>
+      <c r="B73" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C73" s="13">
-        <v>158006019.52700391</v>
-      </c>
-      <c r="D73" s="13">
+      <c r="C73" s="2">
+        <v>267535969</v>
+      </c>
+      <c r="D73">
         <v>20.52</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A74" s="12">
+      <c r="A74" s="13">
         <v>2042</v>
       </c>
-      <c r="B74" s="14" t="s">
+      <c r="B74" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C74" s="13">
+      <c r="C74" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D74" s="13">
+      <c r="D74">
         <v>29.19</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A75" s="12"/>
-      <c r="B75" s="14" t="s">
+      <c r="A75" s="13"/>
+      <c r="B75" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C75" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D75" s="13">
+      <c r="C75" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D75">
         <v>42.69</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A76" s="12"/>
-      <c r="B76" s="14" t="s">
+      <c r="A76" s="13"/>
+      <c r="B76" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C76" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D76" s="13">
+      <c r="C76" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D76">
         <v>150</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A77" s="12"/>
-      <c r="B77" s="14" t="s">
+      <c r="A77" s="13"/>
+      <c r="B77" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C77" s="13">
-        <v>151603615.61576971</v>
-      </c>
-      <c r="D77" s="13">
+      <c r="C77" s="2">
+        <v>257872875</v>
+      </c>
+      <c r="D77">
         <v>20.52</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A78" s="12">
+      <c r="A78" s="13">
         <v>2043</v>
       </c>
-      <c r="B78" s="14" t="s">
+      <c r="B78" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C78" s="13">
+      <c r="C78" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D78" s="13">
+      <c r="D78">
         <v>29.19</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A79" s="12"/>
-      <c r="B79" s="14" t="s">
+      <c r="A79" s="13"/>
+      <c r="B79" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C79" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D79" s="13">
+      <c r="C79" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D79">
         <v>42.69</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A80" s="12"/>
-      <c r="B80" s="14" t="s">
+      <c r="A80" s="13"/>
+      <c r="B80" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C80" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D80" s="13">
+      <c r="C80" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D80">
         <v>150</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A81" s="12"/>
-      <c r="B81" s="14" t="s">
+      <c r="A81" s="13"/>
+      <c r="B81" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C81" s="13">
-        <v>145460637.11101869</v>
-      </c>
-      <c r="D81" s="13">
+      <c r="C81" s="2">
+        <v>248744486</v>
+      </c>
+      <c r="D81">
         <v>20.52</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A82" s="12">
+      <c r="A82" s="13">
         <v>2044</v>
       </c>
-      <c r="B82" s="14" t="s">
+      <c r="B82" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C82" s="13">
+      <c r="C82" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D82" s="13">
+      <c r="D82">
         <v>29.19</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A83" s="12"/>
-      <c r="B83" s="14" t="s">
+      <c r="A83" s="13"/>
+      <c r="B83" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C83" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D83" s="13">
+      <c r="C83" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D83">
         <v>42.69</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A84" s="12"/>
-      <c r="B84" s="14" t="s">
+      <c r="A84" s="13"/>
+      <c r="B84" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C84" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D84" s="13">
+      <c r="C84" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D84">
         <v>150</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" s="12"/>
-      <c r="B85" s="14" t="s">
+      <c r="A85" s="13"/>
+      <c r="B85" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C85" s="13">
-        <v>139566572.0952802</v>
-      </c>
-      <c r="D85" s="13">
+      <c r="C85" s="2">
+        <v>240136226</v>
+      </c>
+      <c r="D85">
         <v>20.52</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A86" s="12">
+      <c r="A86" s="13">
         <v>2045</v>
       </c>
-      <c r="B86" s="14" t="s">
+      <c r="B86" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C86" s="13">
+      <c r="C86" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D86" s="13">
+      <c r="D86">
         <v>29.19</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A87" s="12"/>
-      <c r="B87" s="14" t="s">
+      <c r="A87" s="13"/>
+      <c r="B87" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C87" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D87" s="13">
+      <c r="C87" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D87">
         <v>42.69</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A88" s="12"/>
-      <c r="B88" s="14" t="s">
+      <c r="A88" s="13"/>
+      <c r="B88" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C88" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D88" s="13">
+      <c r="C88" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D88">
         <v>150</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" s="12"/>
-      <c r="B89" s="14" t="s">
+      <c r="A89" s="13"/>
+      <c r="B89" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C89" s="13">
-        <v>133911334.5939794</v>
-      </c>
-      <c r="D89" s="13">
+      <c r="C89" s="2">
+        <v>232032192</v>
+      </c>
+      <c r="D89">
         <v>20.52</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" s="12">
+      <c r="A90" s="13">
         <v>2046</v>
       </c>
-      <c r="B90" s="14" t="s">
+      <c r="B90" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C90" s="13">
+      <c r="C90" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D90" s="13">
+      <c r="D90">
         <v>29.19</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" s="12"/>
-      <c r="B91" s="14" t="s">
+      <c r="A91" s="13"/>
+      <c r="B91" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C91" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D91" s="13">
+      <c r="C91" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D91">
         <v>42.69</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A92" s="12"/>
-      <c r="B92" s="14" t="s">
+      <c r="A92" s="13"/>
+      <c r="B92" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C92" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D92" s="13">
+      <c r="C92" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D92">
         <v>150</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A93" s="12"/>
-      <c r="B93" s="14" t="s">
+      <c r="A93" s="13"/>
+      <c r="B93" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C93" s="13">
-        <v>128485247.3162314</v>
-      </c>
-      <c r="D93" s="13">
+      <c r="C93" s="2">
+        <v>224418473</v>
+      </c>
+      <c r="D93">
         <v>20.52</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A94" s="12">
+      <c r="A94" s="13">
         <v>2047</v>
       </c>
-      <c r="B94" s="14" t="s">
+      <c r="B94" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C94" s="13">
+      <c r="C94" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D94" s="13">
+      <c r="D94">
         <v>29.19</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" s="12"/>
-      <c r="B95" s="14" t="s">
+      <c r="A95" s="13"/>
+      <c r="B95" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C95" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D95" s="13">
+      <c r="C95" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D95">
         <v>42.69</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A96" s="12"/>
-      <c r="B96" s="14" t="s">
+      <c r="A96" s="13"/>
+      <c r="B96" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C96" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D96" s="13">
+      <c r="C96" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D96">
         <v>150</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A97" s="12"/>
-      <c r="B97" s="14" t="s">
+      <c r="A97" s="13"/>
+      <c r="B97" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C97" s="13">
-        <v>123279025.09497771</v>
-      </c>
-      <c r="D97" s="13">
+      <c r="C97" s="2">
+        <v>217272367</v>
+      </c>
+      <c r="D97">
         <v>20.52</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A98" s="12">
+      <c r="A98" s="13">
         <v>2048</v>
       </c>
-      <c r="B98" s="14" t="s">
+      <c r="B98" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C98" s="13">
+      <c r="C98" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D98" s="13">
+      <c r="D98">
         <v>29.19</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A99" s="12"/>
-      <c r="B99" s="14" t="s">
+      <c r="A99" s="13"/>
+      <c r="B99" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C99" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D99" s="13">
+      <c r="C99" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D99">
         <v>42.69</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A100" s="12"/>
-      <c r="B100" s="14" t="s">
+      <c r="A100" s="13"/>
+      <c r="B100" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C100" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D100" s="13">
+      <c r="C100" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D100">
         <v>150</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A101" s="12"/>
-      <c r="B101" s="14" t="s">
+      <c r="A101" s="13"/>
+      <c r="B101" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C101" s="13">
-        <v>118283758.9981292</v>
-      </c>
-      <c r="D101" s="13">
+      <c r="C101" s="2">
+        <v>210579168</v>
+      </c>
+      <c r="D101">
         <v>20.52</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A102" s="12">
+      <c r="A102" s="13">
         <v>2049</v>
       </c>
-      <c r="B102" s="14" t="s">
+      <c r="B102" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C102" s="13">
+      <c r="C102" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D102" s="13">
+      <c r="D102">
         <v>29.19</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A103" s="12"/>
-      <c r="B103" s="14" t="s">
+      <c r="A103" s="13"/>
+      <c r="B103" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C103" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D103" s="13">
+      <c r="C103" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D103">
         <v>42.69</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A104" s="12"/>
-      <c r="B104" s="14" t="s">
+      <c r="A104" s="13"/>
+      <c r="B104" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C104" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D104" s="13">
+      <c r="C104" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D104">
         <v>150</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A105" s="12"/>
-      <c r="B105" s="14" t="s">
+      <c r="A105" s="13"/>
+      <c r="B105" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C105" s="13">
-        <v>113490901.083525</v>
-      </c>
-      <c r="D105" s="13">
+      <c r="C105" s="2">
+        <v>204325995</v>
+      </c>
+      <c r="D105">
         <v>20.52</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A106" s="12">
+      <c r="A106" s="13">
         <v>2050</v>
       </c>
-      <c r="B106" s="14" t="s">
+      <c r="B106" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="C106" s="13">
+      <c r="C106" s="2">
         <v>270613611.10000002</v>
       </c>
-      <c r="D106" s="13">
+      <c r="D106">
         <v>29.19</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A107" s="12"/>
-      <c r="B107" s="14" t="s">
+      <c r="A107" s="13"/>
+      <c r="B107" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C107" s="13">
-        <v>1047284444.4400001</v>
-      </c>
-      <c r="D107" s="13">
+      <c r="C107" s="2">
+        <v>1047284444</v>
+      </c>
+      <c r="D107">
         <v>42.69</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A108" s="12"/>
-      <c r="B108" s="14" t="s">
+      <c r="A108" s="13"/>
+      <c r="B108" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C108" s="13">
-        <v>2930833333.3299999</v>
-      </c>
-      <c r="D108" s="13">
+      <c r="C108" s="2">
+        <v>2930833333</v>
+      </c>
+      <c r="D108">
         <v>150</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A109" s="12"/>
-      <c r="B109" s="14" t="s">
+      <c r="A109" s="13"/>
+      <c r="B109" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C109" s="13">
-        <v>108892249.7716206</v>
-      </c>
-      <c r="D109" s="13">
+      <c r="C109" s="2">
+        <v>198500000</v>
+      </c>
+      <c r="D109">
         <v>20.52</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B1:B109" xr:uid="{DB5FB19D-A699-4685-BD4E-A72E73D671DD}"/>
   <mergeCells count="27">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A81"/>
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="A82:A85"/>
@@ -12658,6 +12617,26 @@
     <mergeCell ref="A90:A93"/>
     <mergeCell ref="A94:A97"/>
     <mergeCell ref="A98:A101"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A18:A21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>